<commit_message>
Add search bar functionality to only show searched items
</commit_message>
<xml_diff>
--- a/UcuzBilgisayar/BILGISAYAR_URUNLERI.xlsx
+++ b/UcuzBilgisayar/BILGISAYAR_URUNLERI.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/5C3A02D28638C25E/Desktop/ito-bilgisayar-urunleri/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="35" documentId="11_53D540F50A234F1ABE610802856E17AB797854E6" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{194F7FB8-F228-4B16-9FC3-F3A5626F4D8E}"/>
+  <xr:revisionPtr revIDLastSave="1" documentId="11_7309C2F9368B092D02610883D52F35C378783EAB" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{451D7188-90AB-4AA5-91DE-9F1A1FAAFFE0}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="635" uniqueCount="177">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="685" uniqueCount="184">
   <si>
     <t>Ürün adı</t>
   </si>
@@ -37,520 +37,541 @@
     <t>Yorum sayısı</t>
   </si>
   <si>
+    <t>Excalibur E27FVC-E 27" 300HZ 1MS 400NIT Fast VA Curved HDR10 Oyuncu Monitörü</t>
+  </si>
+  <si>
+    <t>Game Garaj Slayer X5T-5050 C7 Intel Core I5 13500HX 16GB Ram 1tb SSD RTX5050 16" Wuxga 165Hz IPS Freedos Oyuncu Laptop</t>
+  </si>
+  <si>
+    <t>Beyaz Oyuncu Masası 160x60, Bilgisayar Masası, Gamer Masası, Gaming Masa, Metal Ayaklı</t>
+  </si>
+  <si>
+    <t>Lenovo LOQ Essential AMD Ryzen 7 7735HS 16GB 512GB SSD RTX3050 Freedos 15.6" FHD 144Hz Taşınabilir Bilgisayar 83S00033TR</t>
+  </si>
+  <si>
+    <t>MSI KATANA 17 HX B14WFK-217TR Intel Core i9 14900HX 32GB 1TB SSD RTX5060 Windows 11 Home 17.3" QHD 240Hz Taşınabilir Bilgisayar</t>
+  </si>
+  <si>
+    <t>Orion Cube 3x Tuştan Değişen RGB Fanlı M-Atx Boş Bilgisayar Kasası Beyaz</t>
+  </si>
+  <si>
+    <t>Lenovo Ideapad Slim 3 AMD Ryzen 7 7735HS 16GB 512GB SSD Freedos 15.3" Taşınabilir Bilgisayar 83K70098TR</t>
+  </si>
+  <si>
+    <t>Apple MacBook Neo A18 Pro 8GB 256GB SSD macOS 13" Taşınabilir Bilgisayar Pastel Pembe  MHFH4TU/A</t>
+  </si>
+  <si>
+    <t>Macbook Air M2 M3 M4 M5 13.6 A3113 A3240 A2681 ile Uyumlu Parlak Simli Şeffaf Kılıf Kapak Koruma</t>
+  </si>
+  <si>
+    <t>IdeaPad Slim3 Intel Core i5-13420H 16GB 512GB SSD 15.3" WUXGA FreeDOS  Dizüstü Bilgisayar 83K1003MTR</t>
+  </si>
+  <si>
+    <t>Yeni 2025 MatePad 11.5" PaperMatte 8GB 256GB Tablet + Klavye</t>
+  </si>
+  <si>
+    <t>Lenovo Ideapad Slim 3 AMD Ryzen 5 7535HS 16GB 512GB SSD Freedos 15.3" Taşınabilir Bilgisayar 83K7009ETR</t>
+  </si>
+  <si>
+    <t>HP AI 15 Intel Core Ultra 5 225U 16GB 512GB SSD Freedos 15.6" Taşınabilir Bilgisayar D51E0EA</t>
+  </si>
+  <si>
+    <t>MSI CYBORG 15 A13UC-2087XTR Intel Core i5 13420H 16GB 512GB SSD RTX3050 Freedos 15.6" FHD 144Hz Taşınabilir Bilgisayar</t>
+  </si>
+  <si>
+    <t>Aspire Lite Intel Celeron-N4500 8GB 256GB SSD 15.6" FHD DOS (İşletim Sistemsiz) Laptop NX.J9SEY.001</t>
+  </si>
+  <si>
+    <t>Asus Zenbook S 16 UM5606WA-RK411W AMD Ryzen AI 9 HX 370 32GB 1TB SSD Windows 11 Home 16" Taşınabilir Bilgisayar</t>
+  </si>
+  <si>
+    <t>Apple MacBook Air M4 16GB 256GB SSD macOS 15" Taşınabilir Bilgisayar Gök Mavisi MC7A4TU/A</t>
+  </si>
+  <si>
+    <t>Pg-46-cl-56 | E414-404-484-474 Renkli Orjinal Kartuş Seti</t>
+  </si>
+  <si>
+    <t>Lenovo LOQE AMD Ryzen 7 7735HS 16GB 512GB SSD RTX4050 Freedos 15.6" Taşınabilir Bilgisayar 83S0002YTR</t>
+  </si>
+  <si>
+    <t>Nirvana Intel Celeron N4020 4GB RAM 120GB SSD Windows 11 Home 15.6" Hd Laptop C370.4020-4C00B</t>
+  </si>
+  <si>
+    <t>Apple MacBook Neo A18 Pro 8GB 512GB SSD macOS 13" Taşınabilir Bilgisayar Indigo MHFG4TU/A</t>
+  </si>
+  <si>
+    <t>Ideapad Slim 3 AMD Ryzen 5-7520U 8GB 512GB SSD 15.6" FHD Dizüstü Bilgisayar 82XQ00RWTX</t>
+  </si>
+  <si>
+    <t>Siyah/Beyaz Oyuncu Masası 60x140 Cm, Beyaz Renk Bilgisayar Masası, Gamer Masası, Gaming Masa</t>
+  </si>
+  <si>
+    <t>ASUS TUF Gaming F16 FX608JMR-RV075 Intel Core i7 14650HX 16GB 1TB SSD RTX5060 Freedos 16" Taşınabilir Bilgisayar</t>
+  </si>
+  <si>
     <t>LOQE AMD Ryzen 7-7735HS 16GB 512GB SSD 15.6" FHD 144Hz RTX4050 6GB FreeDOS Gaming Laptop 83S0002YTR</t>
   </si>
   <si>
+    <t>Apple Macbook Air 13.6 M2 M3 M4 M5 A2681 A3113 A3240 A3449 Kristal Kılıf Şeffaf Tam Koruma Kapak</t>
+  </si>
+  <si>
+    <t>Ideapad Slim 3 Intel N100 4gb Ram 128GB Ssd 15.6'' 82XB009GTX</t>
+  </si>
+  <si>
+    <t>Victus 15-FA2051NT Intel Core i5-14450HX 24G 1TB SSD RTX4050 6GB Freedos 15.6" FHD IPS 144Hz D2QG6EA</t>
+  </si>
+  <si>
+    <t>Apple MacBook Air M4 16GB 512GB SSD macOS 13" Taşınabilir Bilgisayar Gece Yarısı MW133TU/A</t>
+  </si>
+  <si>
+    <t>Apple MacBook Air M5 16GB 512GB SSD macOS 13" Taşınabilir Bilgisayar Gök Mavisi MDHH4TU/A</t>
+  </si>
+  <si>
+    <t>13" MacBook Neo Pastel Pembe 256GB</t>
+  </si>
+  <si>
+    <t>Apple MacBook Air M5 16GB 512GB SSD macOS 15" Taşınabilir Bilgisayar Gece Yarısı MDVH4TU/A</t>
+  </si>
+  <si>
+    <t>Pro MP275W E2 27" 120Hz 1ms FHD Flat IPS Adaptive-Sync Monitör</t>
+  </si>
+  <si>
+    <t>Lenovo Case 15.6" Toploader T210 Taşınabilir Bilgisayar Çantası Siyah GX40Q17229</t>
+  </si>
+  <si>
+    <t>Asus Tuf Gaming F16 FX608JMR-RV078 Intel Core I7 14650HX 32GB 1 Tb SSD RTX5060-8GB 115W Freedos 16" 165Hz Wuxga Taşınabilir Bilgisayar</t>
+  </si>
+  <si>
+    <t>Hp Prelude 15.6" Bilgisayar Çantası Gri 2Z8P4AA</t>
+  </si>
+  <si>
+    <t>Triline Nb F160+FP Gazlı Çift Kol Monitör Standı 17-30" Ekran ve 10-17" Dizüstü Bilgisayar İçin Metal</t>
+  </si>
+  <si>
+    <t>Lenovo IdeaPad Slim 3 Intel Core i5 13420H 16GB 512GB SSD Freedos 15.3" Taşınabilir Bilgisayar 83K1003MTR</t>
+  </si>
+  <si>
+    <t>Game Garaj Slayer X7T-5070 C2 Intel Core i7 14650HX 32GB 1TB SSD RTX5070 16" Qhd+ 180Hz IPS Freedos Gaming Laptop</t>
+  </si>
+  <si>
+    <t>Apple MacBook Neo A18 Pro 8GB 256GB SSD macOS 13" Taşınabilir Bilgisayar Indigo MHFF4TU/A</t>
+  </si>
+  <si>
+    <t>Lenovo Ideapad Slim 3 Intel N100 8GB 128GB SSD Windows 11 Home 15.6" FHD Taşınabilir Bilgisayar 82XB00HMTX</t>
+  </si>
+  <si>
+    <t>MSI CYBORG 15 B13WFKG-495XTR Intel Core i7 13620H 32GB 1TB SSD RTX5060 Freedos 15.6" FHD 144Hz Taşınabilir Bilgisayar</t>
+  </si>
+  <si>
+    <t>Apple MacBook Neo A18 Pro 8GB 512GB SSD macOS 13" Taşınabilir Bilgisayar Gümüş MHFC4TU/A</t>
+  </si>
+  <si>
+    <t>Casper Excalibur G915 Intel Core i7 13620H 32GB 1TB SSD RTX5060 Freedos 16" 165Hz Taşınabilir Bilgisayar G915.1362-DF60X-C</t>
+  </si>
+  <si>
+    <t>Game Garaj Slayer X7T-5060 C2 Intel Core I7 14650HX 32GB Ram 1tb SSD RTX5060 16" Qhd+ 180Hz IPS Freedos Gaming Laptop</t>
+  </si>
+  <si>
+    <t>Apple MacBook Neo A18 Pro 8GB 256GB SSD macOS 13" Taşınabilir Bilgisayar Gümüş MHFA4TU/A</t>
+  </si>
+  <si>
+    <t>Game Garaj Slayer X7T-5070 C7 Intel Core I7 14650HX 16GB Ram 1tb SSD RTX5070 16" Qhd+ 180Hz IPS Freedos Gaming Laptop</t>
+  </si>
+  <si>
+    <t>Asus Tuf Gaming A16 FA608UM-RV130 Amd Ryzen 7 260 16GB 512GB SSD RTX5060-8GB 115W Freedos 16" Wuxga 165Hz Taşınabilir Bilgisayar</t>
+  </si>
+  <si>
+    <t>Lenovo Loq 15IRX10 83JE00JQTR I7-13650HX 16GB Ddr5 1tb SSD RTX5060 8gb Tgp 100W 15.6" IPS 144Hz Freedos</t>
+  </si>
+  <si>
+    <t>Apple MacBook Neo A18 Pro 8GB 256GB SSD macOS 13" Taşınabilir Bilgisayar Puslu Sarı MHFD4TU/A</t>
+  </si>
+  <si>
+    <t>MSI CYBORG 17 B13WFKG-091XTR Intel Core i7 13620H 16GB 1TB SSD RTX5060 Freedos 17.3" FHD 144Hz Taşınabilir Bilgisayar</t>
+  </si>
+  <si>
     <t>MSI CYBORG 15 B13WEKG-613XTR Intel Core I7 13620H 16GB 1TB SSD RTX5050 Freedos 15.6" FHD 144Hz Taşınabilir Bilgisayar</t>
   </si>
   <si>
-    <t>Lenovo LOQ Essential AMD Ryzen 7 7735HS 16GB 512GB SSD RTX3050 Freedos 15.6" FHD 144Hz Taşınabilir Bilgisayar 83S00033TR</t>
-  </si>
-  <si>
-    <t>MSI CYBORG 15 A13UC-2087XTR Intel Core i5 13420H 16GB 512GB SSD RTX3050 Freedos 15.6" FHD 144Hz Taşınabilir Bilgisayar</t>
-  </si>
-  <si>
-    <t>Apple MacBook Neo A18 Pro 8GB 512GB SSD macOS 13" Taşınabilir Bilgisayar Indigo MHFG4TU/A</t>
-  </si>
-  <si>
-    <t>Game Garaj Slayer X7T-5070 C7 Intel Core I7 14650HX 16GB Ram 1tb SSD RTX5070 16" Qhd+ 180Hz IPS Freedos Gaming Laptop</t>
-  </si>
-  <si>
-    <t>Yeni 2025 MatePad 11.5" PaperMatte 8GB 256GB Tablet + Klavye</t>
-  </si>
-  <si>
-    <t>Apple MacBook Neo A18 Pro 8GB 256GB SSD macOS 13" Taşınabilir Bilgisayar Puslu Sarı MHFD4TU/A</t>
-  </si>
-  <si>
-    <t>Apple MacBook Neo A18 Pro 8GB 256GB SSD macOS 13" Taşınabilir Bilgisayar Pastel Pembe  MHFH4TU/A</t>
-  </si>
-  <si>
-    <t>Ideapad Slim 3 AMD Ryzen 5-7520U 8GB 512GB SSD 15.6" FHD Dizüstü Bilgisayar 82XQ00RWTX</t>
-  </si>
-  <si>
-    <t>Pro MP275W E2 27" 120Hz 1ms FHD Flat IPS Adaptive-Sync Monitör</t>
-  </si>
-  <si>
-    <t>IdeaPad Slim3 Intel Core i5-13420H 16GB 512GB SSD 15.3" WUXGA FreeDOS  Dizüstü Bilgisayar 83K1003MTR</t>
-  </si>
-  <si>
-    <t>Dynamic Grey Masajlı Oyuncu Koltuğu</t>
-  </si>
-  <si>
-    <t>Asus Tuf Gaming A16 FA608UM-RV130 Amd Ryzen 7 260 16GB 512GB SSD RTX5060-8GB 115W Freedos 16" Wuxga 165Hz Taşınabilir Bilgisayar</t>
-  </si>
-  <si>
-    <t>MSI CYBORG 17 B13WFKG-091XTR Intel Core i7 13620H 16GB 1TB SSD RTX5060 Freedos 17.3" FHD 144Hz Taşınabilir Bilgisayar</t>
-  </si>
-  <si>
-    <t>Excalibur E27FVC-E 27" 300HZ 1MS 400NIT Fast VA Curved HDR10 Oyuncu Monitörü</t>
-  </si>
-  <si>
-    <t>Asus Tuf Gaming F16 FX608JMR-RV078 Intel Core I7 14650HX 32GB 1 Tb SSD RTX5060-8GB 115W Freedos 16" 165Hz Wuxga Taşınabilir Bilgisayar</t>
-  </si>
-  <si>
-    <t>Lenovo Ideapad Slim 3 AMD Ryzen 7 7735HS 16GB 512GB SSD Freedos 15.3" Taşınabilir Bilgisayar 83K70098TR</t>
-  </si>
-  <si>
-    <t>Lenovo Loq 15IRX10 83JE00JQTR I7-13650HX 16GB Ddr5 1tb SSD RTX5060 8gb Tgp 100W 15.6" IPS 144Hz Freedos</t>
-  </si>
-  <si>
-    <t>Victus 15-FA2051NT Intel Core i5-14450HX 24G 1TB SSD RTX4050 6GB Freedos 15.6" FHD IPS 144Hz D2QG6EA</t>
-  </si>
-  <si>
-    <t>Rion R10 24" 165hz 1ms Fhd Va Curved Gaming Monitör (sıfır Ölü Piksel Garantili)</t>
-  </si>
-  <si>
-    <t>MSI KATANA 17 HX B14WFK-217TR Intel Core i9 14900HX 32GB 1TB SSD RTX5060 Windows 11 Home 17.3" QHD 240Hz Taşınabilir Bilgisayar</t>
-  </si>
-  <si>
-    <t>Aspire Lite Intel Celeron-N4500 8GB 256GB SSD 15.6" FHD DOS (İşletim Sistemsiz) Laptop NX.J9SEY.001</t>
-  </si>
-  <si>
-    <t>Beyaz Oyuncu Masası 160x60, Bilgisayar Masası, Gamer Masası, Gaming Masa, Metal Ayaklı</t>
-  </si>
-  <si>
-    <t>Apple Macbook Air 13.6 M2 M3 M4 M5 A2681 A3113 A3240 A3449 Kristal Kılıf Şeffaf Tam Koruma Kapak</t>
-  </si>
-  <si>
-    <t>ASUS TUF Gaming F16 FX608JMR-RV075 Intel Core i7 14650HX 16GB 1TB SSD RTX5060 Freedos 16" Taşınabilir Bilgisayar</t>
-  </si>
-  <si>
-    <t>Apple MacBook Neo A18 Pro 8GB 256GB SSD macOS 13" Taşınabilir Bilgisayar Gümüş MHFA4TU/A</t>
-  </si>
-  <si>
-    <t>Ideapad Slim 3 Intel N100 4gb Ram 128GB Ssd 15.6'' 82XB009GTX</t>
-  </si>
-  <si>
-    <t>Excalibur G915 i7-13620H 32GB 1TB 8GB RTX5070 165Hz 16" Freedos Gaming Laptop G915.1362-DF70X-C</t>
-  </si>
-  <si>
-    <t>Excalibur G870 i7-13620H 32GB 2TB 115W RTX5060 165Hz 15.6" Freedos Gaming Laptop G870.1362-DX60X-C</t>
-  </si>
-  <si>
-    <t>Asus Zenbook S 16 UM5606WA-RK411W AMD Ryzen AI 9 HX 370 32GB 1TB SSD Windows 11 Home 16" Taşınabilir Bilgisayar</t>
-  </si>
-  <si>
     <t>Seagate 4TB Skyhawk RV ST4000VX016 3.5" 5900Rpm 256 MB 7x24 Güvenlik Hdd (Resmi Distribitör Ürünü)</t>
   </si>
   <si>
-    <t>Lenovo IdeaPad Slim 3 Intel Core i5 13420H 16GB 512GB SSD Freedos 15.3" Taşınabilir Bilgisayar 83K1003MTR</t>
-  </si>
-  <si>
-    <t>Game Garaj Slayer X5T-5050 C7 Intel Core I5 13500HX 16GB Ram 1tb SSD RTX5050 16" Wuxga 165Hz IPS Freedos Oyuncu Laptop</t>
-  </si>
-  <si>
-    <t>Apple MacBook Air M4 16GB 256GB SSD macOS 15" Taşınabilir Bilgisayar Gök Mavisi MC7A4TU/A</t>
-  </si>
-  <si>
-    <t>Apple MacBook Air M5 16GB 512GB SSD macOS 13" Taşınabilir Bilgisayar Gök Mavisi MDHH4TU/A</t>
-  </si>
-  <si>
-    <t>Apple MacBook Neo A18 Pro 8GB 256GB SSD macOS 13" Taşınabilir Bilgisayar Indigo MHFF4TU/A</t>
-  </si>
-  <si>
-    <t>Apple MacBook Air M4 16GB 512GB SSD macOS 13" Taşınabilir Bilgisayar Gece Yarısı MW133TU/A</t>
-  </si>
-  <si>
-    <t>Apple MacBook Neo A18 Pro 8GB 512GB SSD macOS 13" Taşınabilir Bilgisayar Gümüş MHFC4TU/A</t>
-  </si>
-  <si>
-    <t>Casper Excalibur G915 Intel Core i7 13620H 32GB 1TB SSD RTX5060 Freedos 16" 165Hz Taşınabilir Bilgisayar G915.1362-DF60X-C</t>
-  </si>
-  <si>
-    <t>Apple MacBook Air M5 16GB 512GB SSD macOS 15" Taşınabilir Bilgisayar Gece Yarısı MDVH4TU/A</t>
-  </si>
-  <si>
-    <t>Game Garaj Slayer X7T-5060 C2 Intel Core I7 14650HX 32GB Ram 1tb SSD RTX5060 16" Qhd+ 180Hz IPS Freedos Gaming Laptop</t>
-  </si>
-  <si>
-    <t>Lenovo LOQE AMD Ryzen 7 7735HS 16GB 512GB SSD RTX4050 Freedos 15.6" Taşınabilir Bilgisayar 83S0002YTR</t>
-  </si>
-  <si>
-    <t>Lenovo Ideapad Slim 3 Intel N100 8GB 128GB SSD Windows 11 Home 15.6" FHD Taşınabilir Bilgisayar 82XB00HMTX</t>
-  </si>
-  <si>
-    <t>Lenovo Ideapad Slim 3 AMD Ryzen 5 7535HS 16GB 512GB SSD Freedos 15.3" Taşınabilir Bilgisayar 83K7009ETR</t>
-  </si>
-  <si>
-    <t>Triline Nb F160+FP Gazlı Çift Kol Monitör Standı 17-30" Ekran ve 10-17" Dizüstü Bilgisayar İçin Metal</t>
-  </si>
-  <si>
-    <t>HP AI 15 Intel Core Ultra 5 225U 16GB 512GB SSD Freedos 15.6" Taşınabilir Bilgisayar D51E0EA</t>
-  </si>
-  <si>
-    <t>Game Garaj Slayer X7T-5070 C2 Intel Core i7 14650HX 32GB 1TB SSD RTX5070 16" Qhd+ 180Hz IPS Freedos Gaming Laptop</t>
-  </si>
-  <si>
-    <t>Lenovo Case 15.6" Toploader T210 Taşınabilir Bilgisayar Çantası Gri GX40Q17231</t>
-  </si>
-  <si>
-    <t>Hp Prelude 15.6" Bilgisayar Çantası Gri 2Z8P4AA</t>
+    <t>CASPER</t>
+  </si>
+  <si>
+    <t>Game Garaj</t>
+  </si>
+  <si>
+    <t>Flinder</t>
+  </si>
+  <si>
+    <t>Lenovo</t>
   </si>
   <si>
     <t>MSI</t>
   </si>
   <si>
-    <t>Lenovo</t>
+    <t>Next Gaming</t>
   </si>
   <si>
     <t>Apple</t>
   </si>
   <si>
-    <t>Game Garaj</t>
+    <t>Techmaster</t>
+  </si>
+  <si>
+    <t>LENOVO</t>
   </si>
   <si>
     <t>Huawei</t>
   </si>
   <si>
-    <t>Fashcolle</t>
+    <t>HP</t>
+  </si>
+  <si>
+    <t>ACER</t>
   </si>
   <si>
     <t>Asus</t>
   </si>
   <si>
-    <t>CASPER</t>
-  </si>
-  <si>
-    <t>HP</t>
-  </si>
-  <si>
-    <t>James Donkey</t>
-  </si>
-  <si>
-    <t>ACER</t>
-  </si>
-  <si>
-    <t>Flinder</t>
+    <t>Canon</t>
   </si>
   <si>
     <t>ASUS</t>
   </si>
   <si>
+    <t>TEKNETSTORE</t>
+  </si>
+  <si>
+    <t>Hp</t>
+  </si>
+  <si>
+    <t>Triline</t>
+  </si>
+  <si>
+    <t>Casper</t>
+  </si>
+  <si>
     <t>Seagate</t>
   </si>
   <si>
-    <t>Casper</t>
-  </si>
-  <si>
-    <t>Triline</t>
-  </si>
-  <si>
-    <t>37939</t>
+    <t>7899</t>
+  </si>
+  <si>
+    <t>53499</t>
+  </si>
+  <si>
+    <t>2799.90</t>
+  </si>
+  <si>
+    <t>39799</t>
+  </si>
+  <si>
+    <t>92049.16</t>
+  </si>
+  <si>
+    <t>1695</t>
+  </si>
+  <si>
+    <t>30950</t>
+  </si>
+  <si>
+    <t>37875</t>
+  </si>
+  <si>
+    <t>448.41</t>
+  </si>
+  <si>
+    <t>27199</t>
+  </si>
+  <si>
+    <t>13999</t>
+  </si>
+  <si>
+    <t>26989</t>
+  </si>
+  <si>
+    <t>28499</t>
+  </si>
+  <si>
+    <t>35999</t>
+  </si>
+  <si>
+    <t>14199</t>
+  </si>
+  <si>
+    <t>78999</t>
+  </si>
+  <si>
+    <t>66000</t>
+  </si>
+  <si>
+    <t>2006.31</t>
+  </si>
+  <si>
+    <t>39999</t>
+  </si>
+  <si>
+    <t>15006.81</t>
+  </si>
+  <si>
+    <t>43522</t>
+  </si>
+  <si>
+    <t>20949</t>
+  </si>
+  <si>
+    <t>2028</t>
+  </si>
+  <si>
+    <t>69999</t>
+  </si>
+  <si>
+    <t>37999</t>
+  </si>
+  <si>
+    <t>449</t>
+  </si>
+  <si>
+    <t>13480</t>
+  </si>
+  <si>
+    <t>48223.33</t>
+  </si>
+  <si>
+    <t>63662.52</t>
+  </si>
+  <si>
+    <t>80000</t>
+  </si>
+  <si>
+    <t>89000</t>
+  </si>
+  <si>
+    <t>5099</t>
+  </si>
+  <si>
+    <t>537.79</t>
+  </si>
+  <si>
+    <t>74880</t>
+  </si>
+  <si>
+    <t>569</t>
+  </si>
+  <si>
+    <t>4299</t>
+  </si>
+  <si>
+    <t>27399</t>
+  </si>
+  <si>
+    <t>78998.99</t>
+  </si>
+  <si>
+    <t>38225</t>
+  </si>
+  <si>
+    <t>16699</t>
+  </si>
+  <si>
+    <t>62261</t>
+  </si>
+  <si>
+    <t>48990</t>
+  </si>
+  <si>
+    <t>64599</t>
+  </si>
+  <si>
+    <t>70998.99</t>
+  </si>
+  <si>
+    <t>38949</t>
+  </si>
+  <si>
+    <t>54942.26</t>
+  </si>
+  <si>
+    <t>61599</t>
+  </si>
+  <si>
+    <t>42800</t>
+  </si>
+  <si>
+    <t>58299</t>
   </si>
   <si>
     <t>50420</t>
   </si>
   <si>
-    <t>39799</t>
-  </si>
-  <si>
-    <t>35999</t>
-  </si>
-  <si>
-    <t>43577.82</t>
-  </si>
-  <si>
-    <t>70998.99</t>
-  </si>
-  <si>
-    <t>13999</t>
-  </si>
-  <si>
-    <t>42800</t>
-  </si>
-  <si>
-    <t>37994</t>
-  </si>
-  <si>
-    <t>20949</t>
-  </si>
-  <si>
-    <t>5099</t>
-  </si>
-  <si>
-    <t>27249</t>
-  </si>
-  <si>
-    <t>4649</t>
-  </si>
-  <si>
-    <t>55470.17</t>
-  </si>
-  <si>
-    <t>58299</t>
-  </si>
-  <si>
-    <t>7899</t>
-  </si>
-  <si>
-    <t>75899</t>
-  </si>
-  <si>
-    <t>30950</t>
-  </si>
-  <si>
-    <t>61350.47</t>
-  </si>
-  <si>
-    <t>48223.33</t>
-  </si>
-  <si>
-    <t>3289</t>
-  </si>
-  <si>
-    <t>92049.16</t>
-  </si>
-  <si>
-    <t>14199</t>
-  </si>
-  <si>
-    <t>2799.90</t>
-  </si>
-  <si>
-    <t>449</t>
-  </si>
-  <si>
-    <t>69999</t>
-  </si>
-  <si>
-    <t>38950</t>
-  </si>
-  <si>
-    <t>13480</t>
-  </si>
-  <si>
-    <t>87949</t>
-  </si>
-  <si>
-    <t>68137.94</t>
-  </si>
-  <si>
-    <t>78999</t>
-  </si>
-  <si>
-    <t>7850</t>
-  </si>
-  <si>
-    <t>28999</t>
-  </si>
-  <si>
-    <t>53499</t>
-  </si>
-  <si>
-    <t>58999</t>
-  </si>
-  <si>
-    <t>79500</t>
-  </si>
-  <si>
-    <t>38505.48</t>
-  </si>
-  <si>
-    <t>63662.52</t>
-  </si>
-  <si>
-    <t>43932.01</t>
-  </si>
-  <si>
-    <t>64599</t>
-  </si>
-  <si>
-    <t>89999</t>
-  </si>
-  <si>
-    <t>71386.10</t>
-  </si>
-  <si>
-    <t>39999</t>
-  </si>
-  <si>
-    <t>16949</t>
-  </si>
-  <si>
-    <t>26999</t>
-  </si>
-  <si>
-    <t>4299</t>
-  </si>
-  <si>
-    <t>28499</t>
-  </si>
-  <si>
-    <t>78998.99</t>
-  </si>
-  <si>
-    <t>481.54</t>
-  </si>
-  <si>
-    <t>569</t>
+    <t>7954</t>
+  </si>
+  <si>
+    <t>4.3/5</t>
+  </si>
+  <si>
+    <t>4.8/5</t>
+  </si>
+  <si>
+    <t>4.6/5</t>
+  </si>
+  <si>
+    <t>4.9/5</t>
+  </si>
+  <si>
+    <t>5.0/5</t>
+  </si>
+  <si>
+    <t>4.2/5</t>
+  </si>
+  <si>
+    <t>4.5/5</t>
+  </si>
+  <si>
+    <t>4.4/5</t>
+  </si>
+  <si>
+    <t>3.1/5</t>
   </si>
   <si>
     <t>4.1/5</t>
   </si>
   <si>
+    <t>4.0/5</t>
+  </si>
+  <si>
+    <t>5/5</t>
+  </si>
+  <si>
     <t>4.7/5</t>
   </si>
   <si>
-    <t>4.6/5</t>
-  </si>
-  <si>
-    <t>4.9/5</t>
-  </si>
-  <si>
-    <t>4.5/5</t>
-  </si>
-  <si>
-    <t>4.8/5</t>
-  </si>
-  <si>
-    <t>4.4/5</t>
-  </si>
-  <si>
-    <t>4.2/5</t>
-  </si>
-  <si>
-    <t>4.3/5</t>
-  </si>
-  <si>
-    <t>5/5</t>
-  </si>
-  <si>
-    <t>4.0/5</t>
-  </si>
-  <si>
-    <t>3.1/5</t>
+    <t>369</t>
+  </si>
+  <si>
+    <t>51</t>
+  </si>
+  <si>
+    <t>143</t>
+  </si>
+  <si>
+    <t>11</t>
+  </si>
+  <si>
+    <t>40</t>
+  </si>
+  <si>
+    <t>23</t>
+  </si>
+  <si>
+    <t>94</t>
+  </si>
+  <si>
+    <t>19</t>
+  </si>
+  <si>
+    <t>1</t>
+  </si>
+  <si>
+    <t>111</t>
+  </si>
+  <si>
+    <t>124</t>
+  </si>
+  <si>
+    <t>28</t>
+  </si>
+  <si>
+    <t>46</t>
+  </si>
+  <si>
+    <t>10</t>
+  </si>
+  <si>
+    <t>44</t>
+  </si>
+  <si>
+    <t>17</t>
+  </si>
+  <si>
+    <t>92</t>
+  </si>
+  <si>
+    <t>1019</t>
+  </si>
+  <si>
+    <t>21</t>
+  </si>
+  <si>
+    <t>14</t>
+  </si>
+  <si>
+    <t>29</t>
+  </si>
+  <si>
+    <t>31</t>
   </si>
   <si>
     <t>9</t>
   </si>
   <si>
+    <t>1959</t>
+  </si>
+  <si>
+    <t>1160</t>
+  </si>
+  <si>
+    <t>4</t>
+  </si>
+  <si>
+    <t>283</t>
+  </si>
+  <si>
+    <t>8</t>
+  </si>
+  <si>
+    <t>39</t>
+  </si>
+  <si>
+    <t>6</t>
+  </si>
+  <si>
+    <t>24</t>
+  </si>
+  <si>
+    <t>2747</t>
+  </si>
+  <si>
+    <t>123</t>
+  </si>
+  <si>
+    <t>134</t>
+  </si>
+  <si>
+    <t>152</t>
+  </si>
+  <si>
     <t>18</t>
   </si>
   <si>
-    <t>11</t>
-  </si>
-  <si>
-    <t>10</t>
-  </si>
-  <si>
-    <t>21</t>
+    <t>114</t>
+  </si>
+  <si>
+    <t>238</t>
   </si>
   <si>
     <t>32</t>
   </si>
   <si>
-    <t>124</t>
-  </si>
-  <si>
-    <t>23</t>
-  </si>
-  <si>
-    <t>19</t>
-  </si>
-  <si>
-    <t>14</t>
-  </si>
-  <si>
-    <t>24</t>
-  </si>
-  <si>
-    <t>111</t>
-  </si>
-  <si>
-    <t>5789</t>
-  </si>
-  <si>
-    <t>6</t>
+    <t>27</t>
   </si>
   <si>
     <t>58</t>
   </si>
   <si>
-    <t>369</t>
-  </si>
-  <si>
-    <t>29</t>
-  </si>
-  <si>
-    <t>93</t>
-  </si>
-  <si>
-    <t>27</t>
-  </si>
-  <si>
-    <t>4</t>
-  </si>
-  <si>
-    <t>213</t>
-  </si>
-  <si>
-    <t>39</t>
-  </si>
-  <si>
-    <t>44</t>
-  </si>
-  <si>
-    <t>143</t>
-  </si>
-  <si>
-    <t>1959</t>
-  </si>
-  <si>
-    <t>31</t>
-  </si>
-  <si>
-    <t>1160</t>
-  </si>
-  <si>
-    <t>26</t>
-  </si>
-  <si>
-    <t>36</t>
-  </si>
-  <si>
-    <t>17</t>
-  </si>
-  <si>
     <t>99</t>
-  </si>
-  <si>
-    <t>134</t>
-  </si>
-  <si>
-    <t>51</t>
-  </si>
-  <si>
-    <t>92</t>
-  </si>
-  <si>
-    <t>8</t>
-  </si>
-  <si>
-    <t>28</t>
-  </si>
-  <si>
-    <t>282</t>
-  </si>
-  <si>
-    <t>114</t>
-  </si>
-  <si>
-    <t>238</t>
-  </si>
-  <si>
-    <t>46</t>
-  </si>
-  <si>
-    <t>152</t>
-  </si>
-  <si>
-    <t>2747</t>
-  </si>
-  <si>
-    <t>123</t>
-  </si>
-  <si>
-    <t>Acer</t>
   </si>
 </sst>
 </file>
@@ -603,10 +624,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -896,11 +913,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F127"/>
+  <dimension ref="A1:F137"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="2" max="2" width="122" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.6328125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.35">
@@ -928,16 +944,16 @@
         <v>5</v>
       </c>
       <c r="C2" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="D2" t="s">
-        <v>71</v>
+        <v>78</v>
       </c>
       <c r="E2" t="s">
-        <v>121</v>
+        <v>129</v>
       </c>
       <c r="F2" t="s">
-        <v>133</v>
+        <v>142</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.35">
@@ -948,16 +964,16 @@
         <v>6</v>
       </c>
       <c r="C3" t="s">
-        <v>55</v>
+        <v>59</v>
       </c>
       <c r="D3" t="s">
-        <v>72</v>
+        <v>79</v>
       </c>
       <c r="E3" t="s">
-        <v>122</v>
+        <v>130</v>
       </c>
       <c r="F3" t="s">
-        <v>134</v>
+        <v>143</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.35">
@@ -968,16 +984,16 @@
         <v>7</v>
       </c>
       <c r="C4" t="s">
-        <v>56</v>
+        <v>60</v>
       </c>
       <c r="D4" t="s">
-        <v>73</v>
+        <v>80</v>
       </c>
       <c r="E4" t="s">
-        <v>123</v>
+        <v>129</v>
       </c>
       <c r="F4" t="s">
-        <v>135</v>
+        <v>144</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.35">
@@ -988,16 +1004,16 @@
         <v>8</v>
       </c>
       <c r="C5" t="s">
-        <v>55</v>
+        <v>61</v>
       </c>
       <c r="D5" t="s">
-        <v>74</v>
+        <v>81</v>
       </c>
       <c r="E5" t="s">
-        <v>124</v>
+        <v>131</v>
       </c>
       <c r="F5" t="s">
-        <v>136</v>
+        <v>145</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.35">
@@ -1008,16 +1024,16 @@
         <v>9</v>
       </c>
       <c r="C6" t="s">
-        <v>57</v>
+        <v>62</v>
       </c>
       <c r="D6" t="s">
-        <v>75</v>
+        <v>82</v>
       </c>
       <c r="E6" t="s">
-        <v>125</v>
+        <v>129</v>
       </c>
       <c r="F6" t="s">
-        <v>137</v>
+        <v>146</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.35">
@@ -1025,19 +1041,19 @@
         <v>5</v>
       </c>
       <c r="B7" t="s">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="C7" t="s">
-        <v>56</v>
+        <v>63</v>
       </c>
       <c r="D7" t="s">
-        <v>73</v>
+        <v>83</v>
       </c>
       <c r="E7" t="s">
-        <v>123</v>
+        <v>130</v>
       </c>
       <c r="F7" t="s">
-        <v>135</v>
+        <v>147</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.35">
@@ -1045,19 +1061,19 @@
         <v>6</v>
       </c>
       <c r="B8" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="C8" t="s">
-        <v>58</v>
+        <v>61</v>
       </c>
       <c r="D8" t="s">
-        <v>76</v>
+        <v>84</v>
       </c>
       <c r="E8" t="s">
-        <v>126</v>
+        <v>131</v>
       </c>
       <c r="F8" t="s">
-        <v>138</v>
+        <v>148</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.35">
@@ -1065,19 +1081,19 @@
         <v>7</v>
       </c>
       <c r="B9" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="C9" t="s">
-        <v>59</v>
+        <v>64</v>
       </c>
       <c r="D9" t="s">
-        <v>77</v>
+        <v>85</v>
       </c>
       <c r="E9" t="s">
-        <v>125</v>
+        <v>132</v>
       </c>
       <c r="F9" t="s">
-        <v>139</v>
+        <v>149</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.35">
@@ -1085,19 +1101,19 @@
         <v>8</v>
       </c>
       <c r="B10" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="C10" t="s">
-        <v>57</v>
+        <v>65</v>
       </c>
       <c r="D10" t="s">
-        <v>78</v>
+        <v>86</v>
       </c>
       <c r="E10" t="s">
-        <v>126</v>
+        <v>133</v>
       </c>
       <c r="F10" t="s">
-        <v>140</v>
+        <v>150</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.35">
@@ -1105,19 +1121,19 @@
         <v>9</v>
       </c>
       <c r="B11" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C11" t="s">
-        <v>57</v>
+        <v>66</v>
       </c>
       <c r="D11" t="s">
-        <v>79</v>
+        <v>87</v>
       </c>
       <c r="E11" t="s">
-        <v>124</v>
+        <v>134</v>
       </c>
       <c r="F11" t="s">
-        <v>141</v>
+        <v>151</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.35">
@@ -1125,19 +1141,19 @@
         <v>10</v>
       </c>
       <c r="B12" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="C12" t="s">
-        <v>56</v>
+        <v>67</v>
       </c>
       <c r="D12" t="s">
-        <v>80</v>
+        <v>88</v>
       </c>
       <c r="E12" t="s">
-        <v>127</v>
+        <v>135</v>
       </c>
       <c r="F12" t="s">
-        <v>142</v>
+        <v>152</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.35">
@@ -1145,19 +1161,19 @@
         <v>11</v>
       </c>
       <c r="B13" t="s">
-        <v>15</v>
+        <v>9</v>
       </c>
       <c r="C13" t="s">
-        <v>55</v>
+        <v>62</v>
       </c>
       <c r="D13" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="E13" t="s">
-        <v>124</v>
+        <v>129</v>
       </c>
       <c r="F13" t="s">
-        <v>143</v>
+        <v>146</v>
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.35">
@@ -1168,16 +1184,16 @@
         <v>16</v>
       </c>
       <c r="C14" t="s">
-        <v>56</v>
+        <v>61</v>
       </c>
       <c r="D14" t="s">
-        <v>82</v>
+        <v>89</v>
       </c>
       <c r="E14" t="s">
-        <v>128</v>
+        <v>132</v>
       </c>
       <c r="F14" t="s">
-        <v>144</v>
+        <v>153</v>
       </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.35">
@@ -1185,19 +1201,19 @@
         <v>13</v>
       </c>
       <c r="B15" t="s">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="C15" t="s">
-        <v>60</v>
+        <v>64</v>
       </c>
       <c r="D15" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="E15" t="s">
-        <v>129</v>
+        <v>132</v>
       </c>
       <c r="F15" t="s">
-        <v>145</v>
+        <v>149</v>
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.35">
@@ -1205,19 +1221,19 @@
         <v>14</v>
       </c>
       <c r="B16" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C16" t="s">
-        <v>61</v>
+        <v>68</v>
       </c>
       <c r="D16" t="s">
-        <v>84</v>
+        <v>90</v>
       </c>
       <c r="E16" t="s">
-        <v>130</v>
+        <v>136</v>
       </c>
       <c r="F16" t="s">
-        <v>146</v>
+        <v>154</v>
       </c>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.35">
@@ -1225,19 +1241,19 @@
         <v>15</v>
       </c>
       <c r="B17" t="s">
-        <v>11</v>
+        <v>18</v>
       </c>
       <c r="C17" t="s">
-        <v>59</v>
+        <v>62</v>
       </c>
       <c r="D17" t="s">
-        <v>77</v>
+        <v>91</v>
       </c>
       <c r="E17" t="s">
-        <v>125</v>
+        <v>132</v>
       </c>
       <c r="F17" t="s">
-        <v>139</v>
+        <v>155</v>
       </c>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.35">
@@ -1245,19 +1261,19 @@
         <v>16</v>
       </c>
       <c r="B18" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="C18" t="s">
-        <v>61</v>
+        <v>69</v>
       </c>
       <c r="D18" t="s">
-        <v>84</v>
+        <v>92</v>
       </c>
       <c r="E18" t="s">
-        <v>130</v>
+        <v>137</v>
       </c>
       <c r="F18" t="s">
-        <v>146</v>
+        <v>156</v>
       </c>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.35">
@@ -1265,19 +1281,19 @@
         <v>17</v>
       </c>
       <c r="B19" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C19" t="s">
-        <v>55</v>
+        <v>70</v>
       </c>
       <c r="D19" t="s">
-        <v>85</v>
+        <v>93</v>
       </c>
       <c r="E19" t="s">
-        <v>125</v>
+        <v>132</v>
       </c>
       <c r="F19" t="s">
-        <v>147</v>
+        <v>157</v>
       </c>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.35">
@@ -1285,19 +1301,19 @@
         <v>18</v>
       </c>
       <c r="B20" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C20" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="D20" t="s">
-        <v>86</v>
+        <v>94</v>
       </c>
       <c r="E20" t="s">
-        <v>129</v>
+        <v>132</v>
       </c>
       <c r="F20" t="s">
-        <v>148</v>
+        <v>158</v>
       </c>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.35">
@@ -1305,19 +1321,19 @@
         <v>19</v>
       </c>
       <c r="B21" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="C21" t="s">
-        <v>61</v>
+        <v>71</v>
       </c>
       <c r="D21" t="s">
-        <v>87</v>
+        <v>95</v>
       </c>
       <c r="E21" t="s">
-        <v>123</v>
+        <v>133</v>
       </c>
       <c r="F21" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.35">
@@ -1325,19 +1341,19 @@
         <v>20</v>
       </c>
       <c r="B22" t="s">
-        <v>16</v>
+        <v>23</v>
       </c>
       <c r="C22" t="s">
-        <v>56</v>
+        <v>61</v>
       </c>
       <c r="D22" t="s">
-        <v>82</v>
+        <v>96</v>
       </c>
       <c r="E22" t="s">
-        <v>128</v>
+        <v>135</v>
       </c>
       <c r="F22" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.35">
@@ -1345,19 +1361,19 @@
         <v>21</v>
       </c>
       <c r="B23" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="C23" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="D23" t="s">
-        <v>88</v>
+        <v>97</v>
       </c>
       <c r="E23" t="s">
-        <v>123</v>
+        <v>138</v>
       </c>
       <c r="F23" t="s">
-        <v>150</v>
+        <v>159</v>
       </c>
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.35">
@@ -1365,19 +1381,19 @@
         <v>22</v>
       </c>
       <c r="B24" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="C24" t="s">
-        <v>56</v>
+        <v>64</v>
       </c>
       <c r="D24" t="s">
-        <v>89</v>
+        <v>98</v>
       </c>
       <c r="E24" t="s">
-        <v>126</v>
+        <v>135</v>
       </c>
       <c r="F24" t="s">
-        <v>151</v>
+        <v>160</v>
       </c>
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.35">
@@ -1385,19 +1401,19 @@
         <v>23</v>
       </c>
       <c r="B25" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="C25" t="s">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="D25" t="s">
-        <v>90</v>
+        <v>99</v>
       </c>
       <c r="E25" t="s">
-        <v>131</v>
+        <v>136</v>
       </c>
       <c r="F25" t="s">
-        <v>152</v>
+        <v>161</v>
       </c>
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.35">
@@ -1405,19 +1421,19 @@
         <v>24</v>
       </c>
       <c r="B26" t="s">
-        <v>25</v>
+        <v>13</v>
       </c>
       <c r="C26" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="D26" t="s">
-        <v>91</v>
+        <v>86</v>
       </c>
       <c r="E26" t="s">
-        <v>127</v>
+        <v>133</v>
       </c>
       <c r="F26" t="s">
-        <v>153</v>
+        <v>150</v>
       </c>
     </row>
     <row r="27" spans="1:6" x14ac:dyDescent="0.35">
@@ -1425,19 +1441,19 @@
         <v>25</v>
       </c>
       <c r="B27" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="C27" t="s">
-        <v>55</v>
+        <v>60</v>
       </c>
       <c r="D27" t="s">
-        <v>92</v>
+        <v>100</v>
       </c>
       <c r="E27" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="F27" t="s">
-        <v>154</v>
+        <v>162</v>
       </c>
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.35">
@@ -1445,19 +1461,19 @@
         <v>26</v>
       </c>
       <c r="B28" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="C28" t="s">
-        <v>65</v>
+        <v>72</v>
       </c>
       <c r="D28" t="s">
-        <v>93</v>
+        <v>101</v>
       </c>
       <c r="E28" t="s">
-        <v>132</v>
+        <v>135</v>
       </c>
       <c r="F28" t="s">
-        <v>155</v>
+        <v>163</v>
       </c>
     </row>
     <row r="29" spans="1:6" x14ac:dyDescent="0.35">
@@ -1465,19 +1481,19 @@
         <v>27</v>
       </c>
       <c r="B29" t="s">
-        <v>28</v>
+        <v>7</v>
       </c>
       <c r="C29" t="s">
-        <v>66</v>
+        <v>60</v>
       </c>
       <c r="D29" t="s">
-        <v>94</v>
+        <v>80</v>
       </c>
       <c r="E29" t="s">
         <v>129</v>
       </c>
       <c r="F29" t="s">
-        <v>156</v>
+        <v>144</v>
       </c>
     </row>
     <row r="30" spans="1:6" x14ac:dyDescent="0.35">
@@ -1488,16 +1504,16 @@
         <v>29</v>
       </c>
       <c r="C30" t="s">
-        <v>57</v>
+        <v>66</v>
       </c>
       <c r="D30" t="s">
-        <v>95</v>
+        <v>102</v>
       </c>
       <c r="E30" t="s">
-        <v>125</v>
+        <v>138</v>
       </c>
       <c r="F30" t="s">
-        <v>157</v>
+        <v>164</v>
       </c>
     </row>
     <row r="31" spans="1:6" x14ac:dyDescent="0.35">
@@ -1505,19 +1521,19 @@
         <v>29</v>
       </c>
       <c r="B31" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="C31" t="s">
-        <v>67</v>
+        <v>60</v>
       </c>
       <c r="D31" t="s">
-        <v>96</v>
+        <v>100</v>
       </c>
       <c r="E31" t="s">
-        <v>125</v>
+        <v>131</v>
       </c>
       <c r="F31" t="s">
-        <v>158</v>
+        <v>162</v>
       </c>
     </row>
     <row r="32" spans="1:6" x14ac:dyDescent="0.35">
@@ -1525,19 +1541,19 @@
         <v>30</v>
       </c>
       <c r="B32" t="s">
-        <v>17</v>
+        <v>10</v>
       </c>
       <c r="C32" t="s">
-        <v>60</v>
+        <v>63</v>
       </c>
       <c r="D32" t="s">
         <v>83</v>
       </c>
       <c r="E32" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="F32" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
     </row>
     <row r="33" spans="1:6" x14ac:dyDescent="0.35">
@@ -1545,19 +1561,19 @@
         <v>31</v>
       </c>
       <c r="B33" t="s">
-        <v>8</v>
+        <v>30</v>
       </c>
       <c r="C33" t="s">
-        <v>55</v>
+        <v>73</v>
       </c>
       <c r="D33" t="s">
-        <v>74</v>
+        <v>103</v>
       </c>
       <c r="E33" t="s">
-        <v>124</v>
+        <v>135</v>
       </c>
       <c r="F33" t="s">
-        <v>136</v>
+        <v>165</v>
       </c>
     </row>
     <row r="34" spans="1:6" x14ac:dyDescent="0.35">
@@ -1565,19 +1581,19 @@
         <v>32</v>
       </c>
       <c r="B34" t="s">
-        <v>31</v>
+        <v>14</v>
       </c>
       <c r="C34" t="s">
-        <v>57</v>
+        <v>66</v>
       </c>
       <c r="D34" t="s">
-        <v>97</v>
+        <v>87</v>
       </c>
       <c r="E34" t="s">
-        <v>130</v>
+        <v>134</v>
       </c>
       <c r="F34" t="s">
-        <v>135</v>
+        <v>151</v>
       </c>
     </row>
     <row r="35" spans="1:6" x14ac:dyDescent="0.35">
@@ -1585,19 +1601,19 @@
         <v>33</v>
       </c>
       <c r="B35" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C35" t="s">
-        <v>56</v>
+        <v>66</v>
       </c>
       <c r="D35" t="s">
-        <v>98</v>
+        <v>104</v>
       </c>
       <c r="E35" t="s">
-        <v>121</v>
+        <v>138</v>
       </c>
       <c r="F35" t="s">
-        <v>159</v>
+        <v>166</v>
       </c>
     </row>
     <row r="36" spans="1:6" x14ac:dyDescent="0.35">
@@ -1605,19 +1621,19 @@
         <v>34</v>
       </c>
       <c r="B36" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C36" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="D36" t="s">
-        <v>99</v>
+        <v>105</v>
       </c>
       <c r="E36" t="s">
-        <v>131</v>
+        <v>139</v>
       </c>
       <c r="F36" t="s">
-        <v>160</v>
+        <v>167</v>
       </c>
     </row>
     <row r="37" spans="1:6" x14ac:dyDescent="0.35">
@@ -1625,19 +1641,19 @@
         <v>35</v>
       </c>
       <c r="B37" t="s">
-        <v>34</v>
+        <v>15</v>
       </c>
       <c r="C37" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="D37" t="s">
-        <v>100</v>
+        <v>88</v>
       </c>
       <c r="E37" t="s">
-        <v>125</v>
+        <v>135</v>
       </c>
       <c r="F37" t="s">
-        <v>161</v>
+        <v>152</v>
       </c>
     </row>
     <row r="38" spans="1:6" x14ac:dyDescent="0.35">
@@ -1645,19 +1661,19 @@
         <v>36</v>
       </c>
       <c r="B38" t="s">
-        <v>25</v>
+        <v>33</v>
       </c>
       <c r="C38" t="s">
         <v>64</v>
       </c>
       <c r="D38" t="s">
-        <v>91</v>
+        <v>106</v>
       </c>
       <c r="E38" t="s">
-        <v>127</v>
+        <v>130</v>
       </c>
       <c r="F38" t="s">
-        <v>153</v>
+        <v>168</v>
       </c>
     </row>
     <row r="39" spans="1:6" x14ac:dyDescent="0.35">
@@ -1665,19 +1681,19 @@
         <v>37</v>
       </c>
       <c r="B39" t="s">
-        <v>35</v>
+        <v>24</v>
       </c>
       <c r="C39" t="s">
-        <v>61</v>
+        <v>58</v>
       </c>
       <c r="D39" t="s">
-        <v>101</v>
+        <v>97</v>
       </c>
       <c r="E39" t="s">
-        <v>124</v>
+        <v>138</v>
       </c>
       <c r="F39" t="s">
-        <v>162</v>
+        <v>159</v>
       </c>
     </row>
     <row r="40" spans="1:6" x14ac:dyDescent="0.35">
@@ -1685,19 +1701,19 @@
         <v>38</v>
       </c>
       <c r="B40" t="s">
-        <v>5</v>
+        <v>34</v>
       </c>
       <c r="C40" t="s">
-        <v>56</v>
+        <v>64</v>
       </c>
       <c r="D40" t="s">
-        <v>71</v>
+        <v>107</v>
       </c>
       <c r="E40" t="s">
-        <v>121</v>
+        <v>135</v>
       </c>
       <c r="F40" t="s">
-        <v>133</v>
+        <v>169</v>
       </c>
     </row>
     <row r="41" spans="1:6" x14ac:dyDescent="0.35">
@@ -1705,19 +1721,19 @@
         <v>39</v>
       </c>
       <c r="B41" t="s">
-        <v>14</v>
+        <v>35</v>
       </c>
       <c r="C41" t="s">
-        <v>56</v>
+        <v>64</v>
       </c>
       <c r="D41" t="s">
-        <v>80</v>
+        <v>85</v>
       </c>
       <c r="E41" t="s">
-        <v>127</v>
+        <v>131</v>
       </c>
       <c r="F41" t="s">
-        <v>142</v>
+        <v>170</v>
       </c>
     </row>
     <row r="42" spans="1:6" x14ac:dyDescent="0.35">
@@ -1725,19 +1741,19 @@
         <v>40</v>
       </c>
       <c r="B42" t="s">
-        <v>13</v>
+        <v>19</v>
       </c>
       <c r="C42" t="s">
-        <v>57</v>
+        <v>69</v>
       </c>
       <c r="D42" t="s">
-        <v>79</v>
+        <v>92</v>
       </c>
       <c r="E42" t="s">
-        <v>124</v>
+        <v>137</v>
       </c>
       <c r="F42" t="s">
-        <v>141</v>
+        <v>156</v>
       </c>
     </row>
     <row r="43" spans="1:6" x14ac:dyDescent="0.35">
@@ -1745,19 +1761,19 @@
         <v>41</v>
       </c>
       <c r="B43" t="s">
-        <v>15</v>
+        <v>36</v>
       </c>
       <c r="C43" t="s">
-        <v>55</v>
+        <v>64</v>
       </c>
       <c r="D43" t="s">
-        <v>81</v>
+        <v>108</v>
       </c>
       <c r="E43" t="s">
-        <v>124</v>
+        <v>140</v>
       </c>
       <c r="F43" t="s">
-        <v>143</v>
+        <v>171</v>
       </c>
     </row>
     <row r="44" spans="1:6" x14ac:dyDescent="0.35">
@@ -1765,19 +1781,19 @@
         <v>42</v>
       </c>
       <c r="B44" t="s">
-        <v>11</v>
+        <v>37</v>
       </c>
       <c r="C44" t="s">
-        <v>59</v>
+        <v>62</v>
       </c>
       <c r="D44" t="s">
-        <v>77</v>
+        <v>109</v>
       </c>
       <c r="E44" t="s">
-        <v>125</v>
+        <v>132</v>
       </c>
       <c r="F44" t="s">
-        <v>139</v>
+        <v>172</v>
       </c>
     </row>
     <row r="45" spans="1:6" x14ac:dyDescent="0.35">
@@ -1785,19 +1801,19 @@
         <v>43</v>
       </c>
       <c r="B45" t="s">
-        <v>26</v>
+        <v>22</v>
       </c>
       <c r="C45" t="s">
-        <v>55</v>
+        <v>71</v>
       </c>
       <c r="D45" t="s">
-        <v>92</v>
+        <v>95</v>
       </c>
       <c r="E45" t="s">
-        <v>129</v>
+        <v>133</v>
       </c>
       <c r="F45" t="s">
-        <v>154</v>
+        <v>150</v>
       </c>
     </row>
     <row r="46" spans="1:6" x14ac:dyDescent="0.35">
@@ -1805,19 +1821,19 @@
         <v>44</v>
       </c>
       <c r="B46" t="s">
-        <v>20</v>
+        <v>38</v>
       </c>
       <c r="C46" t="s">
-        <v>69</v>
+        <v>61</v>
       </c>
       <c r="D46" t="s">
-        <v>86</v>
+        <v>110</v>
       </c>
       <c r="E46" t="s">
-        <v>129</v>
+        <v>141</v>
       </c>
       <c r="F46" t="s">
-        <v>148</v>
+        <v>173</v>
       </c>
     </row>
     <row r="47" spans="1:6" x14ac:dyDescent="0.35">
@@ -1825,19 +1841,19 @@
         <v>45</v>
       </c>
       <c r="B47" t="s">
-        <v>24</v>
+        <v>39</v>
       </c>
       <c r="C47" t="s">
-        <v>63</v>
+        <v>70</v>
       </c>
       <c r="D47" t="s">
-        <v>90</v>
+        <v>111</v>
       </c>
       <c r="E47" t="s">
         <v>131</v>
       </c>
       <c r="F47" t="s">
-        <v>152</v>
+        <v>162</v>
       </c>
     </row>
     <row r="48" spans="1:6" x14ac:dyDescent="0.35">
@@ -1845,19 +1861,19 @@
         <v>46</v>
       </c>
       <c r="B48" t="s">
-        <v>16</v>
+        <v>40</v>
       </c>
       <c r="C48" t="s">
-        <v>56</v>
+        <v>74</v>
       </c>
       <c r="D48" t="s">
-        <v>82</v>
+        <v>112</v>
       </c>
       <c r="E48" t="s">
-        <v>128</v>
+        <v>141</v>
       </c>
       <c r="F48" t="s">
-        <v>144</v>
+        <v>174</v>
       </c>
     </row>
     <row r="49" spans="1:6" x14ac:dyDescent="0.35">
@@ -1865,19 +1881,19 @@
         <v>47</v>
       </c>
       <c r="B49" t="s">
-        <v>36</v>
+        <v>5</v>
       </c>
       <c r="C49" t="s">
-        <v>68</v>
+        <v>58</v>
       </c>
       <c r="D49" t="s">
-        <v>102</v>
+        <v>78</v>
       </c>
       <c r="E49" t="s">
         <v>129</v>
       </c>
       <c r="F49" t="s">
-        <v>163</v>
+        <v>142</v>
       </c>
     </row>
     <row r="50" spans="1:6" x14ac:dyDescent="0.35">
@@ -1885,19 +1901,19 @@
         <v>48</v>
       </c>
       <c r="B50" t="s">
-        <v>27</v>
+        <v>41</v>
       </c>
       <c r="C50" t="s">
-        <v>65</v>
+        <v>75</v>
       </c>
       <c r="D50" t="s">
-        <v>93</v>
+        <v>113</v>
       </c>
       <c r="E50" t="s">
         <v>132</v>
       </c>
       <c r="F50" t="s">
-        <v>155</v>
+        <v>163</v>
       </c>
     </row>
     <row r="51" spans="1:6" x14ac:dyDescent="0.35">
@@ -1905,19 +1921,19 @@
         <v>49</v>
       </c>
       <c r="B51" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="C51" t="s">
-        <v>57</v>
+        <v>66</v>
       </c>
       <c r="D51" t="s">
-        <v>95</v>
+        <v>99</v>
       </c>
       <c r="E51" t="s">
-        <v>125</v>
+        <v>136</v>
       </c>
       <c r="F51" t="s">
-        <v>157</v>
+        <v>161</v>
       </c>
     </row>
     <row r="52" spans="1:6" x14ac:dyDescent="0.35">
@@ -1925,19 +1941,19 @@
         <v>50</v>
       </c>
       <c r="B52" t="s">
-        <v>28</v>
+        <v>7</v>
       </c>
       <c r="C52" t="s">
-        <v>66</v>
+        <v>60</v>
       </c>
       <c r="D52" t="s">
-        <v>94</v>
+        <v>80</v>
       </c>
       <c r="E52" t="s">
         <v>129</v>
       </c>
       <c r="F52" t="s">
-        <v>156</v>
+        <v>144</v>
       </c>
     </row>
     <row r="53" spans="1:6" x14ac:dyDescent="0.35">
@@ -1945,19 +1961,19 @@
         <v>51</v>
       </c>
       <c r="B53" t="s">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="C53" t="s">
-        <v>60</v>
+        <v>65</v>
       </c>
       <c r="D53" t="s">
-        <v>83</v>
+        <v>86</v>
       </c>
       <c r="E53" t="s">
-        <v>129</v>
+        <v>133</v>
       </c>
       <c r="F53" t="s">
-        <v>145</v>
+        <v>150</v>
       </c>
     </row>
     <row r="54" spans="1:6" x14ac:dyDescent="0.35">
@@ -1965,19 +1981,19 @@
         <v>52</v>
       </c>
       <c r="B54" t="s">
-        <v>32</v>
+        <v>10</v>
       </c>
       <c r="C54" t="s">
-        <v>56</v>
+        <v>63</v>
       </c>
       <c r="D54" t="s">
-        <v>98</v>
+        <v>83</v>
       </c>
       <c r="E54" t="s">
-        <v>121</v>
+        <v>130</v>
       </c>
       <c r="F54" t="s">
-        <v>159</v>
+        <v>147</v>
       </c>
     </row>
     <row r="55" spans="1:6" x14ac:dyDescent="0.35">
@@ -1985,19 +2001,19 @@
         <v>53</v>
       </c>
       <c r="B55" t="s">
-        <v>34</v>
+        <v>42</v>
       </c>
       <c r="C55" t="s">
-        <v>69</v>
+        <v>61</v>
       </c>
       <c r="D55" t="s">
-        <v>100</v>
+        <v>114</v>
       </c>
       <c r="E55" t="s">
-        <v>125</v>
+        <v>135</v>
       </c>
       <c r="F55" t="s">
-        <v>161</v>
+        <v>175</v>
       </c>
     </row>
     <row r="56" spans="1:6" x14ac:dyDescent="0.35">
@@ -2005,19 +2021,19 @@
         <v>54</v>
       </c>
       <c r="B56" t="s">
-        <v>33</v>
+        <v>29</v>
       </c>
       <c r="C56" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="D56" t="s">
-        <v>99</v>
+        <v>102</v>
       </c>
       <c r="E56" t="s">
-        <v>131</v>
+        <v>138</v>
       </c>
       <c r="F56" t="s">
-        <v>160</v>
+        <v>164</v>
       </c>
     </row>
     <row r="57" spans="1:6" x14ac:dyDescent="0.35">
@@ -2025,19 +2041,19 @@
         <v>55</v>
       </c>
       <c r="B57" t="s">
-        <v>25</v>
+        <v>14</v>
       </c>
       <c r="C57" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="D57" t="s">
-        <v>91</v>
+        <v>87</v>
       </c>
       <c r="E57" t="s">
-        <v>127</v>
+        <v>134</v>
       </c>
       <c r="F57" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
     </row>
     <row r="58" spans="1:6" x14ac:dyDescent="0.35">
@@ -2045,19 +2061,19 @@
         <v>56</v>
       </c>
       <c r="B58" t="s">
-        <v>5</v>
+        <v>27</v>
       </c>
       <c r="C58" t="s">
-        <v>56</v>
+        <v>60</v>
       </c>
       <c r="D58" t="s">
-        <v>71</v>
+        <v>100</v>
       </c>
       <c r="E58" t="s">
-        <v>121</v>
+        <v>131</v>
       </c>
       <c r="F58" t="s">
-        <v>133</v>
+        <v>162</v>
       </c>
     </row>
     <row r="59" spans="1:6" x14ac:dyDescent="0.35">
@@ -2065,19 +2081,19 @@
         <v>57</v>
       </c>
       <c r="B59" t="s">
-        <v>15</v>
+        <v>30</v>
       </c>
       <c r="C59" t="s">
-        <v>55</v>
+        <v>73</v>
       </c>
       <c r="D59" t="s">
-        <v>81</v>
+        <v>103</v>
       </c>
       <c r="E59" t="s">
-        <v>124</v>
+        <v>135</v>
       </c>
       <c r="F59" t="s">
-        <v>143</v>
+        <v>165</v>
       </c>
     </row>
     <row r="60" spans="1:6" x14ac:dyDescent="0.35">
@@ -2085,19 +2101,19 @@
         <v>58</v>
       </c>
       <c r="B60" t="s">
-        <v>37</v>
+        <v>28</v>
       </c>
       <c r="C60" t="s">
-        <v>56</v>
+        <v>72</v>
       </c>
       <c r="D60" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="E60" t="s">
-        <v>125</v>
+        <v>135</v>
       </c>
       <c r="F60" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
     </row>
     <row r="61" spans="1:6" x14ac:dyDescent="0.35">
@@ -2105,19 +2121,19 @@
         <v>59</v>
       </c>
       <c r="B61" t="s">
-        <v>20</v>
+        <v>43</v>
       </c>
       <c r="C61" t="s">
-        <v>69</v>
+        <v>59</v>
       </c>
       <c r="D61" t="s">
-        <v>86</v>
+        <v>115</v>
       </c>
       <c r="E61" t="s">
-        <v>129</v>
+        <v>135</v>
       </c>
       <c r="F61" t="s">
-        <v>148</v>
+        <v>176</v>
       </c>
     </row>
     <row r="62" spans="1:6" x14ac:dyDescent="0.35">
@@ -2125,19 +2141,19 @@
         <v>60</v>
       </c>
       <c r="B62" t="s">
-        <v>16</v>
+        <v>44</v>
       </c>
       <c r="C62" t="s">
-        <v>56</v>
+        <v>64</v>
       </c>
       <c r="D62" t="s">
-        <v>82</v>
+        <v>116</v>
       </c>
       <c r="E62" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="F62" t="s">
-        <v>144</v>
+        <v>153</v>
       </c>
     </row>
     <row r="63" spans="1:6" x14ac:dyDescent="0.35">
@@ -2145,19 +2161,19 @@
         <v>61</v>
       </c>
       <c r="B63" t="s">
-        <v>19</v>
+        <v>23</v>
       </c>
       <c r="C63" t="s">
-        <v>55</v>
+        <v>61</v>
       </c>
       <c r="D63" t="s">
-        <v>85</v>
+        <v>96</v>
       </c>
       <c r="E63" t="s">
-        <v>125</v>
+        <v>135</v>
       </c>
       <c r="F63" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
     </row>
     <row r="64" spans="1:6" x14ac:dyDescent="0.35">
@@ -2165,19 +2181,19 @@
         <v>62</v>
       </c>
       <c r="B64" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="C64" t="s">
-        <v>176</v>
+        <v>66</v>
       </c>
       <c r="D64" t="s">
-        <v>93</v>
+        <v>104</v>
       </c>
       <c r="E64" t="s">
-        <v>132</v>
+        <v>138</v>
       </c>
       <c r="F64" t="s">
-        <v>155</v>
+        <v>166</v>
       </c>
     </row>
     <row r="65" spans="1:6" x14ac:dyDescent="0.35">
@@ -2185,19 +2201,19 @@
         <v>63</v>
       </c>
       <c r="B65" t="s">
-        <v>28</v>
+        <v>45</v>
       </c>
       <c r="C65" t="s">
-        <v>66</v>
+        <v>61</v>
       </c>
       <c r="D65" t="s">
-        <v>94</v>
+        <v>117</v>
       </c>
       <c r="E65" t="s">
         <v>129</v>
       </c>
       <c r="F65" t="s">
-        <v>156</v>
+        <v>163</v>
       </c>
     </row>
     <row r="66" spans="1:6" x14ac:dyDescent="0.35">
@@ -2205,19 +2221,19 @@
         <v>64</v>
       </c>
       <c r="B66" t="s">
-        <v>17</v>
+        <v>11</v>
       </c>
       <c r="C66" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="D66" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="E66" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="F66" t="s">
-        <v>145</v>
+        <v>148</v>
       </c>
     </row>
     <row r="67" spans="1:6" x14ac:dyDescent="0.35">
@@ -2225,19 +2241,19 @@
         <v>65</v>
       </c>
       <c r="B67" t="s">
-        <v>38</v>
+        <v>46</v>
       </c>
       <c r="C67" t="s">
-        <v>58</v>
+        <v>62</v>
       </c>
       <c r="D67" t="s">
-        <v>104</v>
+        <v>118</v>
       </c>
       <c r="E67" t="s">
-        <v>126</v>
+        <v>130</v>
       </c>
       <c r="F67" t="s">
-        <v>165</v>
+        <v>163</v>
       </c>
     </row>
     <row r="68" spans="1:6" x14ac:dyDescent="0.35">
@@ -2245,19 +2261,19 @@
         <v>66</v>
       </c>
       <c r="B68" t="s">
-        <v>31</v>
+        <v>21</v>
       </c>
       <c r="C68" t="s">
-        <v>57</v>
+        <v>64</v>
       </c>
       <c r="D68" t="s">
-        <v>97</v>
+        <v>94</v>
       </c>
       <c r="E68" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="F68" t="s">
-        <v>135</v>
+        <v>158</v>
       </c>
     </row>
     <row r="69" spans="1:6" x14ac:dyDescent="0.35">
@@ -2265,19 +2281,19 @@
         <v>67</v>
       </c>
       <c r="B69" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C69" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="D69" t="s">
-        <v>99</v>
+        <v>105</v>
       </c>
       <c r="E69" t="s">
-        <v>131</v>
+        <v>139</v>
       </c>
       <c r="F69" t="s">
-        <v>160</v>
+        <v>167</v>
       </c>
     </row>
     <row r="70" spans="1:6" x14ac:dyDescent="0.35">
@@ -2285,16 +2301,16 @@
         <v>68</v>
       </c>
       <c r="B70" t="s">
-        <v>25</v>
+        <v>16</v>
       </c>
       <c r="C70" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="D70" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="E70" t="s">
-        <v>127</v>
+        <v>132</v>
       </c>
       <c r="F70" t="s">
         <v>153</v>
@@ -2305,19 +2321,19 @@
         <v>69</v>
       </c>
       <c r="B71" t="s">
-        <v>39</v>
+        <v>15</v>
       </c>
       <c r="C71" t="s">
-        <v>57</v>
+        <v>67</v>
       </c>
       <c r="D71" t="s">
-        <v>105</v>
+        <v>88</v>
       </c>
       <c r="E71" t="s">
-        <v>124</v>
+        <v>135</v>
       </c>
       <c r="F71" t="s">
-        <v>166</v>
+        <v>152</v>
       </c>
     </row>
     <row r="72" spans="1:6" x14ac:dyDescent="0.35">
@@ -2325,19 +2341,19 @@
         <v>70</v>
       </c>
       <c r="B72" t="s">
-        <v>40</v>
+        <v>47</v>
       </c>
       <c r="C72" t="s">
-        <v>57</v>
+        <v>64</v>
       </c>
       <c r="D72" t="s">
-        <v>106</v>
+        <v>119</v>
       </c>
       <c r="E72" t="s">
-        <v>125</v>
+        <v>132</v>
       </c>
       <c r="F72" t="s">
-        <v>167</v>
+        <v>177</v>
       </c>
     </row>
     <row r="73" spans="1:6" x14ac:dyDescent="0.35">
@@ -2345,19 +2361,19 @@
         <v>71</v>
       </c>
       <c r="B73" t="s">
-        <v>41</v>
+        <v>24</v>
       </c>
       <c r="C73" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="D73" t="s">
-        <v>107</v>
+        <v>97</v>
       </c>
       <c r="E73" t="s">
-        <v>126</v>
+        <v>138</v>
       </c>
       <c r="F73" t="s">
-        <v>168</v>
+        <v>159</v>
       </c>
     </row>
     <row r="74" spans="1:6" x14ac:dyDescent="0.35">
@@ -2365,19 +2381,19 @@
         <v>72</v>
       </c>
       <c r="B74" t="s">
-        <v>42</v>
+        <v>48</v>
       </c>
       <c r="C74" t="s">
-        <v>57</v>
+        <v>76</v>
       </c>
       <c r="D74" t="s">
-        <v>108</v>
+        <v>120</v>
       </c>
       <c r="E74" t="s">
-        <v>126</v>
+        <v>135</v>
       </c>
       <c r="F74" t="s">
-        <v>169</v>
+        <v>178</v>
       </c>
     </row>
     <row r="75" spans="1:6" x14ac:dyDescent="0.35">
@@ -2385,19 +2401,19 @@
         <v>73</v>
       </c>
       <c r="B75" t="s">
-        <v>43</v>
+        <v>33</v>
       </c>
       <c r="C75" t="s">
-        <v>57</v>
+        <v>64</v>
       </c>
       <c r="D75" t="s">
-        <v>109</v>
+        <v>106</v>
       </c>
       <c r="E75" t="s">
-        <v>124</v>
+        <v>130</v>
       </c>
       <c r="F75" t="s">
-        <v>134</v>
+        <v>168</v>
       </c>
     </row>
     <row r="76" spans="1:6" x14ac:dyDescent="0.35">
@@ -2408,16 +2424,16 @@
         <v>44</v>
       </c>
       <c r="C76" t="s">
-        <v>69</v>
+        <v>64</v>
       </c>
       <c r="D76" t="s">
-        <v>110</v>
+        <v>116</v>
       </c>
       <c r="E76" t="s">
-        <v>125</v>
+        <v>130</v>
       </c>
       <c r="F76" t="s">
-        <v>170</v>
+        <v>153</v>
       </c>
     </row>
     <row r="77" spans="1:6" x14ac:dyDescent="0.35">
@@ -2425,19 +2441,19 @@
         <v>75</v>
       </c>
       <c r="B77" t="s">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="C77" t="s">
-        <v>57</v>
+        <v>76</v>
       </c>
       <c r="D77" t="s">
-        <v>111</v>
+        <v>120</v>
       </c>
       <c r="E77" t="s">
-        <v>130</v>
+        <v>135</v>
       </c>
       <c r="F77" t="s">
-        <v>146</v>
+        <v>178</v>
       </c>
     </row>
     <row r="78" spans="1:6" x14ac:dyDescent="0.35">
@@ -2445,19 +2461,19 @@
         <v>76</v>
       </c>
       <c r="B78" t="s">
-        <v>46</v>
+        <v>26</v>
       </c>
       <c r="C78" t="s">
-        <v>58</v>
+        <v>66</v>
       </c>
       <c r="D78" t="s">
-        <v>76</v>
+        <v>99</v>
       </c>
       <c r="E78" t="s">
-        <v>123</v>
+        <v>136</v>
       </c>
       <c r="F78" t="s">
-        <v>171</v>
+        <v>161</v>
       </c>
     </row>
     <row r="79" spans="1:6" x14ac:dyDescent="0.35">
@@ -2465,19 +2481,19 @@
         <v>77</v>
       </c>
       <c r="B79" t="s">
-        <v>30</v>
+        <v>42</v>
       </c>
       <c r="C79" t="s">
-        <v>67</v>
+        <v>61</v>
       </c>
       <c r="D79" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="E79" t="s">
-        <v>125</v>
+        <v>135</v>
       </c>
       <c r="F79" t="s">
-        <v>158</v>
+        <v>175</v>
       </c>
     </row>
     <row r="80" spans="1:6" x14ac:dyDescent="0.35">
@@ -2485,19 +2501,19 @@
         <v>78</v>
       </c>
       <c r="B80" t="s">
-        <v>47</v>
+        <v>13</v>
       </c>
       <c r="C80" t="s">
-        <v>56</v>
+        <v>65</v>
       </c>
       <c r="D80" t="s">
-        <v>113</v>
+        <v>86</v>
       </c>
       <c r="E80" t="s">
-        <v>125</v>
+        <v>133</v>
       </c>
       <c r="F80" t="s">
-        <v>135</v>
+        <v>150</v>
       </c>
     </row>
     <row r="81" spans="1:6" x14ac:dyDescent="0.35">
@@ -2505,19 +2521,19 @@
         <v>79</v>
       </c>
       <c r="B81" t="s">
-        <v>22</v>
+        <v>34</v>
       </c>
       <c r="C81" t="s">
-        <v>56</v>
+        <v>64</v>
       </c>
       <c r="D81" t="s">
-        <v>88</v>
+        <v>107</v>
       </c>
       <c r="E81" t="s">
-        <v>123</v>
+        <v>135</v>
       </c>
       <c r="F81" t="s">
-        <v>150</v>
+        <v>169</v>
       </c>
     </row>
     <row r="82" spans="1:6" x14ac:dyDescent="0.35">
@@ -2525,19 +2541,19 @@
         <v>80</v>
       </c>
       <c r="B82" t="s">
-        <v>14</v>
+        <v>35</v>
       </c>
       <c r="C82" t="s">
-        <v>56</v>
+        <v>64</v>
       </c>
       <c r="D82" t="s">
-        <v>80</v>
+        <v>85</v>
       </c>
       <c r="E82" t="s">
-        <v>127</v>
+        <v>131</v>
       </c>
       <c r="F82" t="s">
-        <v>142</v>
+        <v>170</v>
       </c>
     </row>
     <row r="83" spans="1:6" x14ac:dyDescent="0.35">
@@ -2545,19 +2561,19 @@
         <v>81</v>
       </c>
       <c r="B83" t="s">
-        <v>9</v>
+        <v>49</v>
       </c>
       <c r="C83" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="D83" t="s">
-        <v>75</v>
+        <v>121</v>
       </c>
       <c r="E83" t="s">
-        <v>125</v>
+        <v>131</v>
       </c>
       <c r="F83" t="s">
-        <v>137</v>
+        <v>179</v>
       </c>
     </row>
     <row r="84" spans="1:6" x14ac:dyDescent="0.35">
@@ -2565,19 +2581,19 @@
         <v>82</v>
       </c>
       <c r="B84" t="s">
-        <v>48</v>
+        <v>43</v>
       </c>
       <c r="C84" t="s">
-        <v>56</v>
+        <v>59</v>
       </c>
       <c r="D84" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="E84" t="s">
-        <v>129</v>
+        <v>135</v>
       </c>
       <c r="F84" t="s">
-        <v>158</v>
+        <v>176</v>
       </c>
     </row>
     <row r="85" spans="1:6" x14ac:dyDescent="0.35">
@@ -2585,19 +2601,19 @@
         <v>83</v>
       </c>
       <c r="B85" t="s">
-        <v>49</v>
+        <v>29</v>
       </c>
       <c r="C85" t="s">
-        <v>56</v>
+        <v>66</v>
       </c>
       <c r="D85" t="s">
-        <v>115</v>
+        <v>102</v>
       </c>
       <c r="E85" t="s">
-        <v>124</v>
+        <v>138</v>
       </c>
       <c r="F85" t="s">
-        <v>168</v>
+        <v>164</v>
       </c>
     </row>
     <row r="86" spans="1:6" x14ac:dyDescent="0.35">
@@ -2605,19 +2621,19 @@
         <v>84</v>
       </c>
       <c r="B86" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="C86" t="s">
-        <v>56</v>
+        <v>64</v>
       </c>
       <c r="D86" t="s">
-        <v>114</v>
+        <v>119</v>
       </c>
       <c r="E86" t="s">
-        <v>129</v>
+        <v>132</v>
       </c>
       <c r="F86" t="s">
-        <v>158</v>
+        <v>177</v>
       </c>
     </row>
     <row r="87" spans="1:6" x14ac:dyDescent="0.35">
@@ -2625,19 +2641,19 @@
         <v>85</v>
       </c>
       <c r="B87" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="C87" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="D87" t="s">
-        <v>90</v>
+        <v>100</v>
       </c>
       <c r="E87" t="s">
         <v>131</v>
       </c>
       <c r="F87" t="s">
-        <v>152</v>
+        <v>162</v>
       </c>
     </row>
     <row r="88" spans="1:6" x14ac:dyDescent="0.35">
@@ -2645,19 +2661,19 @@
         <v>86</v>
       </c>
       <c r="B88" t="s">
-        <v>41</v>
+        <v>50</v>
       </c>
       <c r="C88" t="s">
-        <v>57</v>
+        <v>64</v>
       </c>
       <c r="D88" t="s">
-        <v>107</v>
+        <v>122</v>
       </c>
       <c r="E88" t="s">
-        <v>126</v>
+        <v>140</v>
       </c>
       <c r="F88" t="s">
-        <v>168</v>
+        <v>145</v>
       </c>
     </row>
     <row r="89" spans="1:6" x14ac:dyDescent="0.35">
@@ -2665,19 +2681,19 @@
         <v>87</v>
       </c>
       <c r="B89" t="s">
-        <v>46</v>
+        <v>39</v>
       </c>
       <c r="C89" t="s">
-        <v>58</v>
+        <v>70</v>
       </c>
       <c r="D89" t="s">
-        <v>76</v>
+        <v>111</v>
       </c>
       <c r="E89" t="s">
-        <v>123</v>
+        <v>131</v>
       </c>
       <c r="F89" t="s">
-        <v>171</v>
+        <v>162</v>
       </c>
     </row>
     <row r="90" spans="1:6" x14ac:dyDescent="0.35">
@@ -2685,19 +2701,19 @@
         <v>88</v>
       </c>
       <c r="B90" t="s">
-        <v>29</v>
+        <v>19</v>
       </c>
       <c r="C90" t="s">
-        <v>57</v>
+        <v>69</v>
       </c>
       <c r="D90" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="E90" t="s">
-        <v>125</v>
+        <v>137</v>
       </c>
       <c r="F90" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
     </row>
     <row r="91" spans="1:6" x14ac:dyDescent="0.35">
@@ -2705,16 +2721,16 @@
         <v>89</v>
       </c>
       <c r="B91" t="s">
-        <v>38</v>
+        <v>30</v>
       </c>
       <c r="C91" t="s">
-        <v>58</v>
+        <v>73</v>
       </c>
       <c r="D91" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="E91" t="s">
-        <v>126</v>
+        <v>135</v>
       </c>
       <c r="F91" t="s">
         <v>165</v>
@@ -2725,19 +2741,19 @@
         <v>90</v>
       </c>
       <c r="B92" t="s">
-        <v>33</v>
+        <v>51</v>
       </c>
       <c r="C92" t="s">
-        <v>69</v>
+        <v>59</v>
       </c>
       <c r="D92" t="s">
-        <v>99</v>
+        <v>121</v>
       </c>
       <c r="E92" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="F92" t="s">
-        <v>160</v>
+        <v>180</v>
       </c>
     </row>
     <row r="93" spans="1:6" x14ac:dyDescent="0.35">
@@ -2745,19 +2761,19 @@
         <v>91</v>
       </c>
       <c r="B93" t="s">
-        <v>45</v>
+        <v>52</v>
       </c>
       <c r="C93" t="s">
-        <v>57</v>
+        <v>70</v>
       </c>
       <c r="D93" t="s">
-        <v>111</v>
+        <v>123</v>
       </c>
       <c r="E93" t="s">
-        <v>130</v>
+        <v>140</v>
       </c>
       <c r="F93" t="s">
-        <v>146</v>
+        <v>171</v>
       </c>
     </row>
     <row r="94" spans="1:6" x14ac:dyDescent="0.35">
@@ -2765,19 +2781,19 @@
         <v>92</v>
       </c>
       <c r="B94" t="s">
-        <v>32</v>
+        <v>37</v>
       </c>
       <c r="C94" t="s">
-        <v>56</v>
+        <v>62</v>
       </c>
       <c r="D94" t="s">
-        <v>98</v>
+        <v>109</v>
       </c>
       <c r="E94" t="s">
-        <v>121</v>
+        <v>132</v>
       </c>
       <c r="F94" t="s">
-        <v>159</v>
+        <v>172</v>
       </c>
     </row>
     <row r="95" spans="1:6" x14ac:dyDescent="0.35">
@@ -2785,19 +2801,19 @@
         <v>93</v>
       </c>
       <c r="B95" t="s">
-        <v>21</v>
+        <v>49</v>
       </c>
       <c r="C95" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="D95" t="s">
-        <v>87</v>
+        <v>121</v>
       </c>
       <c r="E95" t="s">
-        <v>123</v>
+        <v>131</v>
       </c>
       <c r="F95" t="s">
-        <v>149</v>
+        <v>179</v>
       </c>
     </row>
     <row r="96" spans="1:6" x14ac:dyDescent="0.35">
@@ -2805,19 +2821,19 @@
         <v>94</v>
       </c>
       <c r="B96" t="s">
-        <v>34</v>
+        <v>22</v>
       </c>
       <c r="C96" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="D96" t="s">
-        <v>100</v>
+        <v>95</v>
       </c>
       <c r="E96" t="s">
-        <v>125</v>
+        <v>133</v>
       </c>
       <c r="F96" t="s">
-        <v>161</v>
+        <v>150</v>
       </c>
     </row>
     <row r="97" spans="1:6" x14ac:dyDescent="0.35">
@@ -2825,19 +2841,19 @@
         <v>95</v>
       </c>
       <c r="B97" t="s">
-        <v>10</v>
+        <v>31</v>
       </c>
       <c r="C97" t="s">
-        <v>58</v>
+        <v>66</v>
       </c>
       <c r="D97" t="s">
-        <v>76</v>
+        <v>104</v>
       </c>
       <c r="E97" t="s">
-        <v>126</v>
+        <v>138</v>
       </c>
       <c r="F97" t="s">
-        <v>138</v>
+        <v>166</v>
       </c>
     </row>
     <row r="98" spans="1:6" x14ac:dyDescent="0.35">
@@ -2845,19 +2861,19 @@
         <v>96</v>
       </c>
       <c r="B98" t="s">
-        <v>37</v>
+        <v>53</v>
       </c>
       <c r="C98" t="s">
-        <v>56</v>
+        <v>61</v>
       </c>
       <c r="D98" t="s">
-        <v>103</v>
+        <v>124</v>
       </c>
       <c r="E98" t="s">
-        <v>125</v>
+        <v>130</v>
       </c>
       <c r="F98" t="s">
-        <v>164</v>
+        <v>181</v>
       </c>
     </row>
     <row r="99" spans="1:6" x14ac:dyDescent="0.35">
@@ -2865,19 +2881,19 @@
         <v>97</v>
       </c>
       <c r="B99" t="s">
-        <v>39</v>
+        <v>50</v>
       </c>
       <c r="C99" t="s">
-        <v>57</v>
+        <v>64</v>
       </c>
       <c r="D99" t="s">
-        <v>105</v>
+        <v>122</v>
       </c>
       <c r="E99" t="s">
-        <v>124</v>
+        <v>140</v>
       </c>
       <c r="F99" t="s">
-        <v>166</v>
+        <v>145</v>
       </c>
     </row>
     <row r="100" spans="1:6" x14ac:dyDescent="0.35">
@@ -2885,19 +2901,19 @@
         <v>98</v>
       </c>
       <c r="B100" t="s">
-        <v>50</v>
+        <v>32</v>
       </c>
       <c r="C100" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="D100" t="s">
-        <v>116</v>
+        <v>105</v>
       </c>
       <c r="E100" t="s">
-        <v>124</v>
+        <v>139</v>
       </c>
       <c r="F100" t="s">
-        <v>158</v>
+        <v>167</v>
       </c>
     </row>
     <row r="101" spans="1:6" x14ac:dyDescent="0.35">
@@ -2905,19 +2921,19 @@
         <v>99</v>
       </c>
       <c r="B101" t="s">
-        <v>14</v>
+        <v>25</v>
       </c>
       <c r="C101" t="s">
-        <v>56</v>
+        <v>64</v>
       </c>
       <c r="D101" t="s">
-        <v>80</v>
+        <v>98</v>
       </c>
       <c r="E101" t="s">
-        <v>127</v>
+        <v>135</v>
       </c>
       <c r="F101" t="s">
-        <v>142</v>
+        <v>160</v>
       </c>
     </row>
     <row r="102" spans="1:6" x14ac:dyDescent="0.35">
@@ -2925,19 +2941,19 @@
         <v>100</v>
       </c>
       <c r="B102" t="s">
-        <v>5</v>
+        <v>15</v>
       </c>
       <c r="C102" t="s">
-        <v>56</v>
+        <v>67</v>
       </c>
       <c r="D102" t="s">
-        <v>71</v>
+        <v>88</v>
       </c>
       <c r="E102" t="s">
-        <v>121</v>
+        <v>135</v>
       </c>
       <c r="F102" t="s">
-        <v>133</v>
+        <v>152</v>
       </c>
     </row>
     <row r="103" spans="1:6" x14ac:dyDescent="0.35">
@@ -2945,19 +2961,19 @@
         <v>101</v>
       </c>
       <c r="B103" t="s">
-        <v>51</v>
+        <v>46</v>
       </c>
       <c r="C103" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="D103" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="E103" t="s">
-        <v>127</v>
+        <v>130</v>
       </c>
       <c r="F103" t="s">
-        <v>172</v>
+        <v>163</v>
       </c>
     </row>
     <row r="104" spans="1:6" x14ac:dyDescent="0.35">
@@ -2965,19 +2981,19 @@
         <v>102</v>
       </c>
       <c r="B104" t="s">
-        <v>52</v>
+        <v>5</v>
       </c>
       <c r="C104" t="s">
         <v>58</v>
       </c>
       <c r="D104" t="s">
-        <v>118</v>
+        <v>78</v>
       </c>
       <c r="E104" t="s">
-        <v>125</v>
+        <v>129</v>
       </c>
       <c r="F104" t="s">
-        <v>173</v>
+        <v>142</v>
       </c>
     </row>
     <row r="105" spans="1:6" x14ac:dyDescent="0.35">
@@ -2985,19 +3001,19 @@
         <v>103</v>
       </c>
       <c r="B105" t="s">
-        <v>11</v>
+        <v>36</v>
       </c>
       <c r="C105" t="s">
-        <v>59</v>
+        <v>64</v>
       </c>
       <c r="D105" t="s">
-        <v>77</v>
+        <v>108</v>
       </c>
       <c r="E105" t="s">
-        <v>125</v>
+        <v>140</v>
       </c>
       <c r="F105" t="s">
-        <v>139</v>
+        <v>171</v>
       </c>
     </row>
     <row r="106" spans="1:6" x14ac:dyDescent="0.35">
@@ -3005,19 +3021,19 @@
         <v>104</v>
       </c>
       <c r="B106" t="s">
-        <v>20</v>
+        <v>7</v>
       </c>
       <c r="C106" t="s">
-        <v>69</v>
+        <v>60</v>
       </c>
       <c r="D106" t="s">
-        <v>86</v>
+        <v>80</v>
       </c>
       <c r="E106" t="s">
         <v>129</v>
       </c>
       <c r="F106" t="s">
-        <v>148</v>
+        <v>144</v>
       </c>
     </row>
     <row r="107" spans="1:6" x14ac:dyDescent="0.35">
@@ -3025,19 +3041,19 @@
         <v>105</v>
       </c>
       <c r="B107" t="s">
-        <v>43</v>
+        <v>54</v>
       </c>
       <c r="C107" t="s">
-        <v>57</v>
+        <v>64</v>
       </c>
       <c r="D107" t="s">
-        <v>109</v>
+        <v>125</v>
       </c>
       <c r="E107" t="s">
-        <v>124</v>
+        <v>130</v>
       </c>
       <c r="F107" t="s">
-        <v>134</v>
+        <v>147</v>
       </c>
     </row>
     <row r="108" spans="1:6" x14ac:dyDescent="0.35">
@@ -3045,19 +3061,19 @@
         <v>106</v>
       </c>
       <c r="B108" t="s">
-        <v>42</v>
+        <v>26</v>
       </c>
       <c r="C108" t="s">
-        <v>57</v>
+        <v>66</v>
       </c>
       <c r="D108" t="s">
-        <v>108</v>
+        <v>99</v>
       </c>
       <c r="E108" t="s">
-        <v>126</v>
+        <v>136</v>
       </c>
       <c r="F108" t="s">
-        <v>169</v>
+        <v>161</v>
       </c>
     </row>
     <row r="109" spans="1:6" x14ac:dyDescent="0.35">
@@ -3065,19 +3081,19 @@
         <v>107</v>
       </c>
       <c r="B109" t="s">
-        <v>24</v>
+        <v>55</v>
       </c>
       <c r="C109" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="D109" t="s">
-        <v>90</v>
+        <v>126</v>
       </c>
       <c r="E109" t="s">
-        <v>131</v>
+        <v>135</v>
       </c>
       <c r="F109" t="s">
-        <v>152</v>
+        <v>182</v>
       </c>
     </row>
     <row r="110" spans="1:6" x14ac:dyDescent="0.35">
@@ -3085,19 +3101,19 @@
         <v>108</v>
       </c>
       <c r="B110" t="s">
-        <v>15</v>
+        <v>56</v>
       </c>
       <c r="C110" t="s">
-        <v>55</v>
+        <v>62</v>
       </c>
       <c r="D110" t="s">
-        <v>81</v>
+        <v>127</v>
       </c>
       <c r="E110" t="s">
-        <v>124</v>
+        <v>141</v>
       </c>
       <c r="F110" t="s">
-        <v>143</v>
+        <v>177</v>
       </c>
     </row>
     <row r="111" spans="1:6" x14ac:dyDescent="0.35">
@@ -3105,19 +3121,19 @@
         <v>109</v>
       </c>
       <c r="B111" t="s">
-        <v>40</v>
+        <v>10</v>
       </c>
       <c r="C111" t="s">
-        <v>57</v>
+        <v>63</v>
       </c>
       <c r="D111" t="s">
-        <v>106</v>
+        <v>83</v>
       </c>
       <c r="E111" t="s">
-        <v>125</v>
+        <v>130</v>
       </c>
       <c r="F111" t="s">
-        <v>167</v>
+        <v>147</v>
       </c>
     </row>
     <row r="112" spans="1:6" x14ac:dyDescent="0.35">
@@ -3125,19 +3141,19 @@
         <v>110</v>
       </c>
       <c r="B112" t="s">
-        <v>23</v>
+        <v>45</v>
       </c>
       <c r="C112" t="s">
-        <v>56</v>
+        <v>61</v>
       </c>
       <c r="D112" t="s">
-        <v>89</v>
+        <v>117</v>
       </c>
       <c r="E112" t="s">
-        <v>126</v>
+        <v>129</v>
       </c>
       <c r="F112" t="s">
-        <v>151</v>
+        <v>163</v>
       </c>
     </row>
     <row r="113" spans="1:6" x14ac:dyDescent="0.35">
@@ -3145,19 +3161,19 @@
         <v>111</v>
       </c>
       <c r="B113" t="s">
-        <v>53</v>
+        <v>30</v>
       </c>
       <c r="C113" t="s">
-        <v>56</v>
+        <v>73</v>
       </c>
       <c r="D113" t="s">
-        <v>119</v>
+        <v>103</v>
       </c>
       <c r="E113" t="s">
-        <v>122</v>
+        <v>135</v>
       </c>
       <c r="F113" t="s">
-        <v>174</v>
+        <v>165</v>
       </c>
     </row>
     <row r="114" spans="1:6" x14ac:dyDescent="0.35">
@@ -3165,19 +3181,19 @@
         <v>112</v>
       </c>
       <c r="B114" t="s">
-        <v>44</v>
+        <v>14</v>
       </c>
       <c r="C114" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="D114" t="s">
-        <v>110</v>
+        <v>87</v>
       </c>
       <c r="E114" t="s">
-        <v>125</v>
+        <v>134</v>
       </c>
       <c r="F114" t="s">
-        <v>170</v>
+        <v>151</v>
       </c>
     </row>
     <row r="115" spans="1:6" x14ac:dyDescent="0.35">
@@ -3188,16 +3204,16 @@
         <v>35</v>
       </c>
       <c r="C115" t="s">
-        <v>61</v>
+        <v>64</v>
       </c>
       <c r="D115" t="s">
-        <v>101</v>
+        <v>85</v>
       </c>
       <c r="E115" t="s">
-        <v>124</v>
+        <v>131</v>
       </c>
       <c r="F115" t="s">
-        <v>162</v>
+        <v>170</v>
       </c>
     </row>
     <row r="116" spans="1:6" x14ac:dyDescent="0.35">
@@ -3205,19 +3221,19 @@
         <v>114</v>
       </c>
       <c r="B116" t="s">
-        <v>29</v>
+        <v>8</v>
       </c>
       <c r="C116" t="s">
-        <v>57</v>
+        <v>61</v>
       </c>
       <c r="D116" t="s">
-        <v>95</v>
+        <v>81</v>
       </c>
       <c r="E116" t="s">
-        <v>125</v>
+        <v>131</v>
       </c>
       <c r="F116" t="s">
-        <v>157</v>
+        <v>145</v>
       </c>
     </row>
     <row r="117" spans="1:6" x14ac:dyDescent="0.35">
@@ -3225,19 +3241,19 @@
         <v>115</v>
       </c>
       <c r="B117" t="s">
-        <v>49</v>
+        <v>56</v>
       </c>
       <c r="C117" t="s">
-        <v>56</v>
+        <v>62</v>
       </c>
       <c r="D117" t="s">
-        <v>115</v>
+        <v>127</v>
       </c>
       <c r="E117" t="s">
-        <v>124</v>
+        <v>141</v>
       </c>
       <c r="F117" t="s">
-        <v>168</v>
+        <v>177</v>
       </c>
     </row>
     <row r="118" spans="1:6" x14ac:dyDescent="0.35">
@@ -3245,19 +3261,19 @@
         <v>116</v>
       </c>
       <c r="B118" t="s">
-        <v>52</v>
+        <v>57</v>
       </c>
       <c r="C118" t="s">
-        <v>58</v>
+        <v>77</v>
       </c>
       <c r="D118" t="s">
-        <v>118</v>
+        <v>128</v>
       </c>
       <c r="E118" t="s">
-        <v>125</v>
+        <v>129</v>
       </c>
       <c r="F118" t="s">
-        <v>173</v>
+        <v>183</v>
       </c>
     </row>
     <row r="119" spans="1:6" x14ac:dyDescent="0.35">
@@ -3265,19 +3281,19 @@
         <v>117</v>
       </c>
       <c r="B119" t="s">
-        <v>51</v>
+        <v>29</v>
       </c>
       <c r="C119" t="s">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="D119" t="s">
-        <v>117</v>
+        <v>102</v>
       </c>
       <c r="E119" t="s">
-        <v>127</v>
+        <v>138</v>
       </c>
       <c r="F119" t="s">
-        <v>172</v>
+        <v>164</v>
       </c>
     </row>
     <row r="120" spans="1:6" x14ac:dyDescent="0.35">
@@ -3285,19 +3301,19 @@
         <v>118</v>
       </c>
       <c r="B120" t="s">
-        <v>6</v>
+        <v>51</v>
       </c>
       <c r="C120" t="s">
-        <v>55</v>
+        <v>59</v>
       </c>
       <c r="D120" t="s">
-        <v>72</v>
+        <v>121</v>
       </c>
       <c r="E120" t="s">
-        <v>122</v>
+        <v>130</v>
       </c>
       <c r="F120" t="s">
-        <v>134</v>
+        <v>180</v>
       </c>
     </row>
     <row r="121" spans="1:6" x14ac:dyDescent="0.35">
@@ -3305,19 +3321,19 @@
         <v>119</v>
       </c>
       <c r="B121" t="s">
-        <v>32</v>
+        <v>54</v>
       </c>
       <c r="C121" t="s">
-        <v>56</v>
+        <v>64</v>
       </c>
       <c r="D121" t="s">
-        <v>98</v>
+        <v>125</v>
       </c>
       <c r="E121" t="s">
-        <v>121</v>
+        <v>130</v>
       </c>
       <c r="F121" t="s">
-        <v>159</v>
+        <v>147</v>
       </c>
     </row>
     <row r="122" spans="1:6" x14ac:dyDescent="0.35">
@@ -3325,19 +3341,19 @@
         <v>120</v>
       </c>
       <c r="B122" t="s">
-        <v>27</v>
+        <v>19</v>
       </c>
       <c r="C122" t="s">
-        <v>65</v>
+        <v>69</v>
       </c>
       <c r="D122" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="E122" t="s">
-        <v>132</v>
+        <v>137</v>
       </c>
       <c r="F122" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
     </row>
     <row r="123" spans="1:6" x14ac:dyDescent="0.35">
@@ -3345,19 +3361,19 @@
         <v>121</v>
       </c>
       <c r="B123" t="s">
-        <v>12</v>
+        <v>18</v>
       </c>
       <c r="C123" t="s">
-        <v>57</v>
+        <v>62</v>
       </c>
       <c r="D123" t="s">
-        <v>78</v>
+        <v>91</v>
       </c>
       <c r="E123" t="s">
-        <v>126</v>
+        <v>132</v>
       </c>
       <c r="F123" t="s">
-        <v>140</v>
+        <v>155</v>
       </c>
     </row>
     <row r="124" spans="1:6" x14ac:dyDescent="0.35">
@@ -3365,19 +3381,19 @@
         <v>122</v>
       </c>
       <c r="B124" t="s">
-        <v>54</v>
+        <v>37</v>
       </c>
       <c r="C124" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="D124" t="s">
-        <v>120</v>
+        <v>109</v>
       </c>
       <c r="E124" t="s">
-        <v>122</v>
+        <v>132</v>
       </c>
       <c r="F124" t="s">
-        <v>175</v>
+        <v>172</v>
       </c>
     </row>
     <row r="125" spans="1:6" x14ac:dyDescent="0.35">
@@ -3385,19 +3401,19 @@
         <v>123</v>
       </c>
       <c r="B125" t="s">
-        <v>34</v>
+        <v>37</v>
       </c>
       <c r="C125" t="s">
-        <v>69</v>
+        <v>62</v>
       </c>
       <c r="D125" t="s">
-        <v>100</v>
+        <v>109</v>
       </c>
       <c r="E125" t="s">
-        <v>125</v>
+        <v>132</v>
       </c>
       <c r="F125" t="s">
-        <v>161</v>
+        <v>172</v>
       </c>
     </row>
     <row r="126" spans="1:6" x14ac:dyDescent="0.35">
@@ -3405,19 +3421,19 @@
         <v>124</v>
       </c>
       <c r="B126" t="s">
-        <v>28</v>
+        <v>53</v>
       </c>
       <c r="C126" t="s">
-        <v>66</v>
+        <v>61</v>
       </c>
       <c r="D126" t="s">
-        <v>94</v>
+        <v>124</v>
       </c>
       <c r="E126" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="F126" t="s">
-        <v>156</v>
+        <v>181</v>
       </c>
     </row>
     <row r="127" spans="1:6" x14ac:dyDescent="0.35">
@@ -3425,19 +3441,219 @@
         <v>125</v>
       </c>
       <c r="B127" t="s">
-        <v>47</v>
+        <v>17</v>
       </c>
       <c r="C127" t="s">
-        <v>56</v>
+        <v>68</v>
       </c>
       <c r="D127" t="s">
-        <v>113</v>
+        <v>90</v>
       </c>
       <c r="E127" t="s">
-        <v>125</v>
+        <v>136</v>
       </c>
       <c r="F127" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="128" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A128">
+        <v>126</v>
+      </c>
+      <c r="B128" t="s">
+        <v>31</v>
+      </c>
+      <c r="C128" t="s">
+        <v>66</v>
+      </c>
+      <c r="D128" t="s">
+        <v>104</v>
+      </c>
+      <c r="E128" t="s">
+        <v>138</v>
+      </c>
+      <c r="F128" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="129" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A129">
+        <v>127</v>
+      </c>
+      <c r="B129" t="s">
+        <v>22</v>
+      </c>
+      <c r="C129" t="s">
+        <v>71</v>
+      </c>
+      <c r="D129" t="s">
+        <v>95</v>
+      </c>
+      <c r="E129" t="s">
+        <v>133</v>
+      </c>
+      <c r="F129" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="130" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A130">
+        <v>128</v>
+      </c>
+      <c r="B130" t="s">
+        <v>52</v>
+      </c>
+      <c r="C130" t="s">
+        <v>70</v>
+      </c>
+      <c r="D130" t="s">
+        <v>123</v>
+      </c>
+      <c r="E130" t="s">
+        <v>140</v>
+      </c>
+      <c r="F130" t="s">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="131" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A131">
+        <v>129</v>
+      </c>
+      <c r="B131" t="s">
+        <v>20</v>
+      </c>
+      <c r="C131" t="s">
+        <v>70</v>
+      </c>
+      <c r="D131" t="s">
+        <v>93</v>
+      </c>
+      <c r="E131" t="s">
+        <v>132</v>
+      </c>
+      <c r="F131" t="s">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="132" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A132">
+        <v>130</v>
+      </c>
+      <c r="B132" t="s">
+        <v>35</v>
+      </c>
+      <c r="C132" t="s">
+        <v>64</v>
+      </c>
+      <c r="D132" t="s">
+        <v>85</v>
+      </c>
+      <c r="E132" t="s">
+        <v>131</v>
+      </c>
+      <c r="F132" t="s">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="133" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A133">
+        <v>131</v>
+      </c>
+      <c r="B133" t="s">
+        <v>55</v>
+      </c>
+      <c r="C133" t="s">
+        <v>62</v>
+      </c>
+      <c r="D133" t="s">
+        <v>126</v>
+      </c>
+      <c r="E133" t="s">
         <v>135</v>
+      </c>
+      <c r="F133" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="134" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A134">
+        <v>132</v>
+      </c>
+      <c r="B134" t="s">
+        <v>6</v>
+      </c>
+      <c r="C134" t="s">
+        <v>59</v>
+      </c>
+      <c r="D134" t="s">
+        <v>79</v>
+      </c>
+      <c r="E134" t="s">
+        <v>130</v>
+      </c>
+      <c r="F134" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="135" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A135">
+        <v>133</v>
+      </c>
+      <c r="B135" t="s">
+        <v>32</v>
+      </c>
+      <c r="C135" t="s">
+        <v>68</v>
+      </c>
+      <c r="D135" t="s">
+        <v>105</v>
+      </c>
+      <c r="E135" t="s">
+        <v>139</v>
+      </c>
+      <c r="F135" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="136" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A136">
+        <v>134</v>
+      </c>
+      <c r="B136" t="s">
+        <v>24</v>
+      </c>
+      <c r="C136" t="s">
+        <v>58</v>
+      </c>
+      <c r="D136" t="s">
+        <v>97</v>
+      </c>
+      <c r="E136" t="s">
+        <v>138</v>
+      </c>
+      <c r="F136" t="s">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="137" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A137">
+        <v>135</v>
+      </c>
+      <c r="B137" t="s">
+        <v>5</v>
+      </c>
+      <c r="C137" t="s">
+        <v>58</v>
+      </c>
+      <c r="D137" t="s">
+        <v>78</v>
+      </c>
+      <c r="E137" t="s">
+        <v>129</v>
+      </c>
+      <c r="F137" t="s">
+        <v>142</v>
       </c>
     </row>
   </sheetData>

</xml_diff>